<commit_message>
vault backup: 2026-07-21 13:55:23
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/MVP功能清单.xlsx
+++ b/公司项目/认知行动/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12420" activeTab="6"/>
+    <workbookView windowWidth="28800" windowHeight="12420" firstSheet="2" activeTab="8"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2529" uniqueCount="955">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2451" uniqueCount="928">
   <si>
     <t>认知行动平台 · 功能清单（V1.0~V1.3）</t>
   </si>
@@ -3196,9 +3196,6 @@
     <t>功能交付阶段排期（12 个月 · 6 人：后端5+前端1）</t>
   </si>
   <si>
-    <t>全量功能分 4 档版本（不砍）。V1.0(4月,第1-4月)演示主链路 / V1.1(3月,第5-7月)线框图补齐 / V1.2(3月,第8-10月)后台增强 / V1.3(2月,第11-12月)深化。阶段按演示主线倒推。完成人代号：后1=MC执行链/后2=MC业务链/后3=SWM+IRS/后4=OCC/后5=COM+DC+OM/前1=前端。</t>
-  </si>
-  <si>
     <t>阶段</t>
   </si>
   <si>
@@ -3211,144 +3208,281 @@
     <t>主要工作</t>
   </si>
   <si>
-    <t>人力分配</t>
-  </si>
-  <si>
     <t>交付物</t>
   </si>
   <si>
     <t>第0阶段·地基</t>
   </si>
   <si>
-    <t>第1-2周</t>
-  </si>
-  <si>
     <t>M0：能登录</t>
   </si>
   <si>
     <t>COM若依原生登录(/login+/getInfo+/getRouters)+Token签发+Redis共享校验+跨控制台SSO；完整RBAC(@PreAuthorize+@DataScope全套)；系统管理控制台11页(若依原生：用户/角色/部门/登录策略/登录日志/菜单/岗位/字典/参数/通知/操作日志)+部门成员管理；5次锁定策略+令牌黑名单；开发环境搭建(K8s/PG/Redis/MinIO)；前端骨架(登录/门户)；MC真机ADB接入打通1台</t>
   </si>
   <si>
-    <t>后5(COM登录+系统管理11页)+前1(骨架+11页)；后1(MC ADB打通)</t>
-  </si>
-  <si>
     <t>可登录的控制台骨架 + 系统管理控制台11页 + 1台真机ADB可见</t>
   </si>
   <si>
     <t>第1阶段·演示灵魂</t>
   </si>
   <si>
-    <t>第3-8周</t>
-  </si>
-  <si>
-    <t>M1：智能体能动★</t>
+    <r>
+      <t>M1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>：智能体能动</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>★</t>
+    </r>
   </si>
   <si>
     <t>IRS部署多模态模型+EI-05接口；MC执行网关收口；agent-runtime调IRS视觉推理→动作→经网关落地；mc-sfu单控WebRTC+宫格；脚本引擎GraalVM。★早期验证点：截图→推理→动作能跑通一次</t>
   </si>
   <si>
-    <t>后3(IRS)+后1(MC执行链/WebRTC)+前1(远控页)</t>
-  </si>
-  <si>
     <t>单台真机：智能体看屏幕自主决策 + WebRTC远控画面</t>
   </si>
   <si>
     <t>第2阶段·提示词供给</t>
   </si>
   <si>
-    <t>第9-12周</t>
-  </si>
-  <si>
-    <t>M2：提示词能驱动</t>
+    <r>
+      <t>M2</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>：提示词能驱动</t>
+    </r>
   </si>
   <si>
     <t>SWM对话编写+swm-gw/swm-memory；提示词包构建；II-14同步MC持存；记忆读写；coze-loop Playground(魔改，时间盒3周)；多台真机(扩到3-8台)宫格同时跑；账号主数据；任务管理；养号节奏</t>
   </si>
   <si>
-    <t>后3(SWM)+后2(MC业务链)+前1(SWM/MC页)</t>
-  </si>
-  <si>
     <t>一群智能体按各自提示词包在多台真机上作业</t>
   </si>
   <si>
-    <t>第3阶段·闭环驱动</t>
-  </si>
-  <si>
-    <t>第13-16周</t>
-  </si>
-  <si>
-    <t>M3：蜂群能编排</t>
+    <r>
+      <t>第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>阶段</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>闭环驱动</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>M3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>：蜂群能编排</t>
+    </r>
   </si>
   <si>
     <t>OCC行动编排轻量版：Web选智能体群+任务→II-10下发MC→效果回传；OCC预设数据看板；DC少量真采集供料；OM最小日志看板(KubeSphere兜底)；全链路联调+演示脚本打磨</t>
   </si>
   <si>
-    <t>后4(OCC)+后5(DC/OM)+前1(OCC/OM页)+全员联调</t>
-  </si>
-  <si>
-    <t>OCC编排驱动蜂群执行 + 效果看板 + 可现场演示的完整系统</t>
-  </si>
-  <si>
-    <t>第4阶段·线框图补齐</t>
-  </si>
-  <si>
-    <t>第5-7月</t>
-  </si>
-  <si>
-    <t>M4：线框图补齐</t>
-  </si>
-  <si>
-    <t>MC补6页(分组/代理池/模板/编排器/IDE/审计)；OCC-13评估；SWM评测3页(评测集/评估器/实验)</t>
-  </si>
-  <si>
-    <t>后1(MC编排/IDE)+后2(MC审计)+后3(SWM评测)+后4(OCC评估)+前1(4页)</t>
-  </si>
-  <si>
-    <t>线框图剩余业务页落地（MC 6 + OCC 1 + SWM 3 = 10页）</t>
+    <r>
+      <t>OCC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>编排驱动蜂群执行</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>效果看板</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>可现场演示的完整系统</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>第</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t>4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>阶段·完善</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>M4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>：脚本编排</t>
+    </r>
+  </si>
+  <si>
+    <t>实现脚本，实现社信信息的用户画面和脚本编排</t>
+  </si>
+  <si>
+    <r>
+      <t>OCC</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>编排脚本</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">+ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>效果看板</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> + </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
+      <t>可现场演示的完整系统</t>
+    </r>
   </si>
   <si>
     <t>第5阶段·后台增强</t>
   </si>
   <si>
-    <t>第8-10月</t>
-  </si>
-  <si>
     <t>M5：后台增强</t>
   </si>
   <si>
     <t>MC桌面端Profile接入+指纹固化+风控对抗；OM指标采集+告警+全文检索；DC调度+代理池+策略自优化；OCC情报分析大脑(4项分析)；SWM记忆沉淀+迭代决策</t>
   </si>
   <si>
-    <t>后1(MC桌面端)+后2(账号深化)+后3(SWM记忆)+后4(OCC情报)+后5(DC/OM)</t>
-  </si>
-  <si>
     <t>后台能力补齐 + 情报分析大脑</t>
   </si>
   <si>
     <t>第6阶段·深化</t>
   </si>
   <si>
-    <t>第11-12月</t>
-  </si>
-  <si>
     <t>M6：深化</t>
   </si>
   <si>
     <t>IRS多模型管理/监控/配额/回退；OCC策略库/内容管理/NebulaGraph图谱/Flowable完整编排</t>
   </si>
   <si>
-    <t>后3(IRS)+后4(OCC深化)</t>
-  </si>
-  <si>
     <t>深化能力落地 + 完整产品形态</t>
   </si>
   <si>
     <t>功能交付风险登记（V1.0~V1.3）</t>
   </si>
   <si>
-    <t>原『降级路径』列改名为『应对·深化路径』——不降级，风险触发后转向后续版本的深化能力承接。</t>
-  </si>
-  <si>
     <t>风险项</t>
   </si>
   <si>
@@ -3415,21 +3549,6 @@
     <t>第3-8周：WebRTC 单控能否出画面</t>
   </si>
   <si>
-    <t>R4</t>
-  </si>
-  <si>
-    <t>范围 vs 时间：全量功能分 4 版本在 12 月 6 人下需控节奏</t>
-  </si>
-  <si>
-    <t>后期质量塌方或版本滑期</t>
-  </si>
-  <si>
-    <t>按版本里程碑评审：V1.0演示主链路必保(MC执行+IRS多模态+SWM提示词包+OCC编排)；V1.1线框图补齐按页优先级；V1.2/V1.3后台增强与深化可按人力弹性调整</t>
-  </si>
-  <si>
-    <t>每个里程碑(M0~M6)评审是否达标</t>
-  </si>
-  <si>
     <t>R5</t>
   </si>
   <si>
@@ -3443,21 +3562,6 @@
   </si>
   <si>
     <t>演示前账号健康检查</t>
-  </si>
-  <si>
-    <t>R6</t>
-  </si>
-  <si>
-    <t>6 人分工单点：后3 兼 SWM+IRS 双主场，负载集中</t>
-  </si>
-  <si>
-    <t>后3 缺勤或瓶颈导致演示灵魂(M1)与提示词供给(M2)双线受阻</t>
-  </si>
-  <si>
-    <t>早期(第1-8周)后3 聚焦IRS+M1验证点，SWM提示词包由后2临时支援；后期(V1.1)SWM评测闭环独立后，后3 可专注IRS深化</t>
-  </si>
-  <si>
-    <t>第3-8周末：IRS+agent-runtime+coze-loop 是否同步推进</t>
   </si>
 </sst>
 </file>
@@ -3471,7 +3575,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="48">
+  <fonts count="47">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3509,10 +3613,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
+      <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3536,11 +3638,6 @@
     <font>
       <sz val="22"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
     <font>
@@ -4137,28 +4234,31 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="43" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="44" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="41" fontId="23" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="24" fillId="0" borderId="0">
+    <xf numFmtId="42" fontId="23" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
@@ -4167,118 +4267,115 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="11" borderId="4">
+    <xf numFmtId="0" fontId="33" fillId="12" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="12" borderId="5">
+    <xf numFmtId="0" fontId="34" fillId="12" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="12" borderId="4">
+    <xf numFmtId="0" fontId="35" fillId="13" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="13" borderId="6">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8">
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="39" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="3" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="36" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="37" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -4300,19 +4397,19 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4339,7 +4436,7 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4348,7 +4445,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -4357,44 +4454,44 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4407,13 +4504,13 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -5053,8 +5150,8 @@
     <tabColor rgb="FFC00000"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15" outlineLevelRow="6" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -5066,152 +5163,110 @@
   <sheetData>
     <row r="1" ht="20.25" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>916</v>
+        <v>900</v>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" spans="1:6">
-      <c r="A2" s="2" t="s">
-        <v>917</v>
-      </c>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" ht="32" customHeight="1" spans="1:6">
       <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>918</v>
+        <v>901</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>919</v>
+        <v>902</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>920</v>
+        <v>903</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>921</v>
+        <v>904</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>922</v>
+        <v>905</v>
       </c>
     </row>
     <row r="4" ht="80" customHeight="1" spans="1:6">
       <c r="A4" s="4" t="s">
-        <v>923</v>
+        <v>906</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>924</v>
+        <v>907</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>925</v>
+        <v>908</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>926</v>
+        <v>909</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>927</v>
+        <v>910</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>928</v>
+        <v>911</v>
       </c>
     </row>
     <row r="5" ht="80" customHeight="1" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>929</v>
+        <v>912</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>930</v>
+        <v>913</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>931</v>
+        <v>914</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>932</v>
+        <v>915</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>933</v>
+        <v>916</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>934</v>
+        <v>917</v>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>935</v>
+        <v>918</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>936</v>
+        <v>919</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>931</v>
+        <v>914</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>937</v>
+        <v>920</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>938</v>
+        <v>921</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>939</v>
+        <v>922</v>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>940</v>
+        <v>923</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>941</v>
+        <v>924</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>931</v>
+        <v>914</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>942</v>
+        <v>925</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>943</v>
+        <v>926</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>944</v>
-      </c>
-    </row>
-    <row r="8" ht="80" customHeight="1" spans="1:6">
-      <c r="A8" s="4" t="s">
-        <v>945</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>946</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>931</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>947</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>948</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>949</v>
-      </c>
-    </row>
-    <row r="9" ht="80" customHeight="1" spans="1:6">
-      <c r="A9" s="4" t="s">
-        <v>950</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>951</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>931</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>952</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>953</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>954</v>
+        <v>927</v>
       </c>
     </row>
   </sheetData>
@@ -7786,9 +7841,7 @@
       <c r="J66" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="K66" s="4">
-        <v>13</v>
-      </c>
+      <c r="K66" s="4"/>
       <c r="L66" s="4"/>
       <c r="M66" s="4" t="s">
         <v>106</v>
@@ -7826,9 +7879,7 @@
       <c r="J67" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="K67" s="4">
-        <v>10</v>
-      </c>
+      <c r="K67" s="4"/>
       <c r="L67" s="4"/>
       <c r="M67" s="4" t="s">
         <v>65</v>
@@ -7866,9 +7917,7 @@
       <c r="J68" s="4" t="s">
         <v>349</v>
       </c>
-      <c r="K68" s="4">
-        <v>13</v>
-      </c>
+      <c r="K68" s="4"/>
       <c r="L68" s="4"/>
       <c r="M68" s="4" t="s">
         <v>65</v>
@@ -7906,9 +7955,7 @@
       <c r="J69" s="4" t="s">
         <v>337</v>
       </c>
-      <c r="K69" s="4">
-        <v>10</v>
-      </c>
+      <c r="K69" s="4"/>
       <c r="L69" s="4"/>
       <c r="M69" s="4" t="s">
         <v>123</v>
@@ -7946,9 +7993,7 @@
       <c r="J70" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="K70" s="4">
-        <v>5</v>
-      </c>
+      <c r="K70" s="4"/>
       <c r="L70" s="4"/>
       <c r="M70" s="4" t="s">
         <v>123</v>
@@ -7986,9 +8031,7 @@
       <c r="J71" s="4" t="s">
         <v>158</v>
       </c>
-      <c r="K71" s="4">
-        <v>8</v>
-      </c>
+      <c r="K71" s="4"/>
       <c r="L71" s="4"/>
       <c r="M71" s="4" t="s">
         <v>65</v>
@@ -8026,9 +8069,7 @@
       <c r="J72" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="K72" s="4">
-        <v>10</v>
-      </c>
+      <c r="K72" s="4"/>
       <c r="L72" s="4"/>
       <c r="M72" s="4" t="s">
         <v>82</v>
@@ -8066,9 +8107,7 @@
       <c r="J73" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="K73" s="4">
-        <v>10</v>
-      </c>
+      <c r="K73" s="4"/>
       <c r="L73" s="4"/>
       <c r="M73" s="4" t="s">
         <v>82</v>
@@ -8106,9 +8145,7 @@
       <c r="J74" s="21" t="s">
         <v>275</v>
       </c>
-      <c r="K74" s="4">
-        <v>13</v>
-      </c>
+      <c r="K74" s="4"/>
       <c r="L74" s="4"/>
       <c r="M74" s="4" t="s">
         <v>82</v>
@@ -8146,9 +8183,7 @@
       <c r="J75" s="4" t="s">
         <v>211</v>
       </c>
-      <c r="K75" s="4">
-        <v>13</v>
-      </c>
+      <c r="K75" s="4"/>
       <c r="L75" s="4"/>
       <c r="M75" s="4" t="s">
         <v>214</v>
@@ -8186,9 +8221,7 @@
       <c r="J76" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="K76" s="14" t="s">
-        <v>65</v>
-      </c>
+      <c r="K76" s="14"/>
       <c r="L76" s="14" t="s">
         <v>65</v>
       </c>
@@ -8228,9 +8261,7 @@
       <c r="J77" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="K77" s="4">
-        <v>10</v>
-      </c>
+      <c r="K77" s="4"/>
       <c r="L77" s="4"/>
       <c r="M77" s="4" t="s">
         <v>204</v>
@@ -8268,9 +8299,7 @@
       <c r="J78" s="4" t="s">
         <v>374</v>
       </c>
-      <c r="K78" s="4">
-        <v>8</v>
-      </c>
+      <c r="K78" s="4"/>
       <c r="L78" s="4"/>
       <c r="M78" s="4" t="s">
         <v>204</v>
@@ -8308,9 +8337,7 @@
       <c r="J79" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="K79" s="4">
-        <v>8</v>
-      </c>
+      <c r="K79" s="4"/>
       <c r="L79" s="4"/>
       <c r="M79" s="4" t="s">
         <v>65</v>
@@ -8348,9 +8375,7 @@
       <c r="J80" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="K80" s="4">
-        <v>5</v>
-      </c>
+      <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4" t="s">
         <v>65</v>
@@ -8388,9 +8413,7 @@
       <c r="J81" s="4" t="s">
         <v>382</v>
       </c>
-      <c r="K81" s="4">
-        <v>8</v>
-      </c>
+      <c r="K81" s="4"/>
       <c r="L81" s="4"/>
       <c r="M81" s="4" t="s">
         <v>65</v>
@@ -8428,9 +8451,7 @@
       <c r="J82" s="4" t="s">
         <v>285</v>
       </c>
-      <c r="K82" s="4">
-        <v>8</v>
-      </c>
+      <c r="K82" s="4"/>
       <c r="L82" s="4"/>
       <c r="M82" s="4" t="s">
         <v>204</v>
@@ -9537,12 +9558,8 @@
       <c r="I10" s="4" t="s">
         <v>472</v>
       </c>
-      <c r="J10" s="4">
-        <v>13</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
       <c r="L10" s="4" t="s">
         <v>65</v>
       </c>
@@ -9619,12 +9636,8 @@
       <c r="I12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="J12" s="4">
-        <v>10</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="J12" s="4"/>
+      <c r="K12" s="4"/>
       <c r="L12" s="4" t="s">
         <v>65</v>
       </c>
@@ -9660,12 +9673,8 @@
       <c r="I13" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="J13" s="4">
-        <v>8</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="J13" s="4"/>
+      <c r="K13" s="4"/>
       <c r="L13" s="4" t="s">
         <v>65</v>
       </c>
@@ -9742,12 +9751,8 @@
       <c r="I15" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="J15" s="4">
-        <v>13</v>
-      </c>
-      <c r="K15" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="J15" s="4"/>
+      <c r="K15" s="20"/>
       <c r="L15" s="4" t="s">
         <v>65</v>
       </c>
@@ -9786,9 +9791,7 @@
       <c r="J16" s="4">
         <v>8</v>
       </c>
-      <c r="K16" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="K16" s="4"/>
       <c r="L16" s="4" t="s">
         <v>65</v>
       </c>
@@ -9829,12 +9832,8 @@
       <c r="I18" s="4" t="s">
         <v>481</v>
       </c>
-      <c r="J18" s="4">
-        <v>10</v>
-      </c>
-      <c r="K18" s="4" t="s">
-        <v>409</v>
-      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
       <c r="L18" s="4" t="s">
         <v>65</v>
       </c>
@@ -12007,7 +12006,7 @@
     <tabColor rgb="FF1F4E79"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M31"/>
+  <dimension ref="A1:L31"/>
   <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -12017,23 +12016,22 @@
     <col min="5" max="5" width="7" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="9" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="9" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customHeight="1" spans="1:13">
+    <row r="1" ht="20.25" customHeight="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>723</v>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1" spans="1:13">
+    <row r="2" ht="40" customHeight="1" spans="1:12">
       <c r="A2" s="18"/>
     </row>
-    <row r="3" ht="32" customHeight="1" spans="1:13">
+    <row r="3" ht="32" customHeight="1" spans="1:12">
       <c r="A3" s="3" t="s">
         <v>44</v>
       </c>
@@ -12056,30 +12054,27 @@
         <v>51</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M3" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1" spans="1:13">
+    <row r="4" ht="40" customHeight="1" spans="1:12">
       <c r="A4" s="13" t="s">
         <v>724</v>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1" spans="1:13">
+    <row r="5" ht="40" customHeight="1" spans="1:12">
       <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
@@ -12102,7 +12097,7 @@
         <v>65</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>65</v>
@@ -12111,16 +12106,13 @@
         <v>65</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M5" s="14" t="s">
         <v>729</v>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1" spans="1:13">
+    <row r="6" ht="40" customHeight="1" spans="1:12">
       <c r="A6" s="4" t="s">
         <v>68</v>
       </c>
@@ -12143,25 +12135,22 @@
         <v>140</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="J6" s="19">
+        <v>65</v>
+      </c>
+      <c r="I6" s="19">
         <v>5</v>
       </c>
-      <c r="K6" s="20" t="s">
+      <c r="J6" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K6" s="4" t="s">
+        <v>734</v>
+      </c>
       <c r="L6" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="M6" s="4" t="s">
         <v>735</v>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1" spans="1:13">
+    <row r="7" ht="40" customHeight="1" spans="1:12">
       <c r="A7" s="4" t="s">
         <v>68</v>
       </c>
@@ -12184,23 +12173,20 @@
         <v>140</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I7" s="4" t="s">
         <v>730</v>
       </c>
-      <c r="J7" s="19"/>
-      <c r="K7" s="20" t="s">
+      <c r="I7" s="19"/>
+      <c r="J7" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K7" s="4" t="s">
+        <v>734</v>
+      </c>
       <c r="L7" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="M7" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" ht="40" customHeight="1" spans="1:13">
+    <row r="8" ht="40" customHeight="1" spans="1:12">
       <c r="A8" s="4" t="s">
         <v>68</v>
       </c>
@@ -12223,23 +12209,20 @@
         <v>140</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I8" s="4" t="s">
         <v>730</v>
       </c>
-      <c r="J8" s="19"/>
-      <c r="K8" s="20" t="s">
+      <c r="I8" s="19"/>
+      <c r="J8" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K8" s="4" t="s">
+        <v>734</v>
+      </c>
       <c r="L8" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="M8" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="40" customHeight="1" spans="1:13">
+    <row r="9" ht="40" customHeight="1" spans="1:12">
       <c r="A9" s="14" t="s">
         <v>59</v>
       </c>
@@ -12262,25 +12245,22 @@
         <v>65</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>66</v>
+        <v>746</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>746</v>
+        <v>65</v>
       </c>
       <c r="J9" s="14" t="s">
         <v>65</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M9" s="14" t="s">
         <v>747</v>
       </c>
     </row>
-    <row r="10" ht="40" customHeight="1" spans="1:13">
+    <row r="10" ht="40" customHeight="1" spans="1:12">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -12303,25 +12283,22 @@
         <v>73</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I10" s="4" t="s">
         <v>297</v>
       </c>
-      <c r="J10" s="19">
+      <c r="I10" s="19">
         <v>14</v>
       </c>
-      <c r="K10" s="20" t="s">
+      <c r="J10" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K10" s="4" t="s">
+        <v>751</v>
+      </c>
       <c r="L10" s="4" t="s">
-        <v>751</v>
-      </c>
-      <c r="M10" s="4" t="s">
         <v>752</v>
       </c>
     </row>
-    <row r="11" ht="40" customHeight="1" spans="1:13">
+    <row r="11" ht="40" customHeight="1" spans="1:12">
       <c r="A11" s="4" t="s">
         <v>68</v>
       </c>
@@ -12344,23 +12321,20 @@
         <v>73</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I11" s="4" t="s">
         <v>748</v>
       </c>
-      <c r="J11" s="19"/>
-      <c r="K11" s="20" t="s">
+      <c r="I11" s="19"/>
+      <c r="J11" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K11" s="4" t="s">
+        <v>756</v>
+      </c>
       <c r="L11" s="4" t="s">
-        <v>756</v>
-      </c>
-      <c r="M11" s="4" t="s">
         <v>757</v>
       </c>
     </row>
-    <row r="12" ht="40" customHeight="1" spans="1:13">
+    <row r="12" ht="40" customHeight="1" spans="1:12">
       <c r="A12" s="4" t="s">
         <v>68</v>
       </c>
@@ -12383,23 +12357,20 @@
         <v>87</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" s="4" t="s">
         <v>753</v>
       </c>
-      <c r="J12" s="19"/>
-      <c r="K12" s="20" t="s">
+      <c r="I12" s="19"/>
+      <c r="J12" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K12" s="4" t="s">
+        <v>756</v>
+      </c>
       <c r="L12" s="4" t="s">
-        <v>756</v>
-      </c>
-      <c r="M12" s="4" t="s">
         <v>760</v>
       </c>
     </row>
-    <row r="13" ht="40" customHeight="1" spans="1:13">
+    <row r="13" ht="40" customHeight="1" spans="1:12">
       <c r="A13" s="21" t="s">
         <v>68</v>
       </c>
@@ -12422,23 +12393,20 @@
         <v>87</v>
       </c>
       <c r="H13" s="21" t="s">
-        <v>304</v>
-      </c>
-      <c r="I13" s="21" t="s">
         <v>730</v>
       </c>
-      <c r="J13" s="19"/>
-      <c r="K13" s="20" t="s">
+      <c r="I13" s="19"/>
+      <c r="J13" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K13" s="4" t="s">
+        <v>764</v>
+      </c>
       <c r="L13" s="4" t="s">
-        <v>764</v>
-      </c>
-      <c r="M13" s="4" t="s">
         <v>765</v>
       </c>
     </row>
-    <row r="14" ht="40" customHeight="1" spans="1:13">
+    <row r="14" ht="40" customHeight="1" spans="1:12">
       <c r="A14" s="14" t="s">
         <v>59</v>
       </c>
@@ -12461,25 +12429,22 @@
         <v>65</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>66</v>
+        <v>753</v>
       </c>
       <c r="I14" s="14" t="s">
-        <v>753</v>
+        <v>65</v>
       </c>
       <c r="J14" s="14" t="s">
         <v>65</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="M14" s="14" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" ht="40" customHeight="1" spans="1:13">
+    </row>
+    <row r="15" ht="40" customHeight="1" spans="1:12">
       <c r="A15" s="4" t="s">
         <v>68</v>
       </c>
@@ -12502,25 +12467,22 @@
         <v>140</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="I15" s="4" t="s">
         <v>753</v>
       </c>
-      <c r="J15" s="19">
+      <c r="I15" s="19">
         <v>5</v>
       </c>
-      <c r="K15" s="20" t="s">
+      <c r="J15" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K15" s="4" t="s">
+        <v>773</v>
+      </c>
       <c r="L15" s="4" t="s">
-        <v>773</v>
-      </c>
-      <c r="M15" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="16" ht="40" customHeight="1" spans="1:13">
+    <row r="16" ht="40" customHeight="1" spans="1:12">
       <c r="A16" s="21" t="s">
         <v>68</v>
       </c>
@@ -12543,23 +12505,20 @@
         <v>140</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I16" s="21" t="s">
         <v>770</v>
       </c>
-      <c r="J16" s="19"/>
-      <c r="K16" s="20" t="s">
+      <c r="I16" s="19"/>
+      <c r="J16" s="20" t="s">
         <v>733</v>
       </c>
+      <c r="K16" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L16" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M16" s="4" t="s">
         <v>777</v>
       </c>
     </row>
-    <row r="17" ht="40" customHeight="1" spans="1:13">
+    <row r="17" ht="40" customHeight="1" spans="1:12">
       <c r="A17" s="14" t="s">
         <v>59</v>
       </c>
@@ -12582,25 +12541,22 @@
         <v>65</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>66</v>
+        <v>770</v>
       </c>
       <c r="I17" s="14" t="s">
-        <v>770</v>
+        <v>65</v>
       </c>
       <c r="J17" s="14" t="s">
         <v>65</v>
       </c>
       <c r="K17" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L17" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M17" s="14" t="s">
         <v>782</v>
       </c>
     </row>
-    <row r="18" ht="40" customHeight="1" spans="1:13">
+    <row r="18" ht="40" customHeight="1" spans="1:12">
       <c r="A18" s="4" t="s">
         <v>68</v>
       </c>
@@ -12621,25 +12577,22 @@
         <v>140</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I18" s="4" t="s">
         <v>770</v>
       </c>
-      <c r="J18" s="19">
+      <c r="I18" s="19">
         <v>10</v>
       </c>
-      <c r="K18" s="20" t="s">
+      <c r="J18" s="20" t="s">
         <v>459</v>
       </c>
+      <c r="K18" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L18" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M18" s="4" t="s">
         <v>786</v>
       </c>
     </row>
-    <row r="19" ht="40" customHeight="1" spans="1:13">
+    <row r="19" ht="40" customHeight="1" spans="1:12">
       <c r="A19" s="4" t="s">
         <v>68</v>
       </c>
@@ -12660,23 +12613,20 @@
         <v>140</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I19" s="4" t="s">
         <v>783</v>
       </c>
-      <c r="J19" s="19"/>
-      <c r="K19" s="20" t="s">
+      <c r="I19" s="19"/>
+      <c r="J19" s="20" t="s">
         <v>459</v>
       </c>
+      <c r="K19" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L19" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M19" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="20" ht="40" customHeight="1" spans="1:13">
+    <row r="20" ht="40" customHeight="1" spans="1:12">
       <c r="A20" s="21" t="s">
         <v>68</v>
       </c>
@@ -12699,23 +12649,20 @@
         <v>140</v>
       </c>
       <c r="H20" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I20" s="21" t="s">
         <v>783</v>
       </c>
-      <c r="J20" s="19"/>
-      <c r="K20" s="20" t="s">
+      <c r="I20" s="19"/>
+      <c r="J20" s="20" t="s">
         <v>459</v>
       </c>
+      <c r="K20" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L20" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M20" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="21" ht="40" customHeight="1" spans="1:13">
+    <row r="21" ht="40" customHeight="1" spans="1:12">
       <c r="A21" s="4" t="s">
         <v>68</v>
       </c>
@@ -12738,23 +12685,20 @@
         <v>140</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I21" s="4" t="s">
         <v>787</v>
       </c>
-      <c r="J21" s="19"/>
-      <c r="K21" s="20" t="s">
+      <c r="I21" s="19"/>
+      <c r="J21" s="20" t="s">
         <v>459</v>
       </c>
+      <c r="K21" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L21" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M21" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="22" ht="40" customHeight="1" spans="1:13">
+    <row r="22" ht="40" customHeight="1" spans="1:12">
       <c r="A22" s="21" t="s">
         <v>68</v>
       </c>
@@ -12776,27 +12720,26 @@
       <c r="G22" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="H22" s="21"/>
-      <c r="I22" s="21" t="s">
+      <c r="H22" s="21" t="s">
         <v>736</v>
       </c>
-      <c r="J22" s="19"/>
-      <c r="K22" s="20" t="s">
+      <c r="I22" s="19"/>
+      <c r="J22" s="20" t="s">
         <v>459</v>
       </c>
+      <c r="K22" s="4" t="s">
+        <v>734</v>
+      </c>
       <c r="L22" s="4" t="s">
-        <v>734</v>
-      </c>
-      <c r="M22" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="23" ht="40" customHeight="1" spans="1:13">
+    <row r="23" ht="40" customHeight="1" spans="1:12">
       <c r="A23" s="17" t="s">
         <v>799</v>
       </c>
     </row>
-    <row r="24" ht="40" customHeight="1" spans="1:13">
+    <row r="24" ht="40" customHeight="1" spans="1:12">
       <c r="A24" s="14" t="s">
         <v>59</v>
       </c>
@@ -12819,7 +12762,7 @@
         <v>65</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I24" s="14" t="s">
         <v>65</v>
@@ -12828,16 +12771,13 @@
         <v>65</v>
       </c>
       <c r="K24" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L24" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M24" s="14" t="s">
         <v>804</v>
       </c>
     </row>
-    <row r="25" ht="40" customHeight="1" spans="1:13">
+    <row r="25" ht="40" customHeight="1" spans="1:12">
       <c r="A25" s="21" t="s">
         <v>68</v>
       </c>
@@ -12860,21 +12800,18 @@
         <v>140</v>
       </c>
       <c r="H25" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I25" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" s="4"/>
-      <c r="K25" s="20"/>
+        <v>65</v>
+      </c>
+      <c r="I25" s="4"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L25" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M25" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="26" ht="40" customHeight="1" spans="1:13">
+    <row r="26" ht="40" customHeight="1" spans="1:12">
       <c r="A26" s="14" t="s">
         <v>59</v>
       </c>
@@ -12897,23 +12834,20 @@
         <v>65</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="I26" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="J26" s="14"/>
+        <v>65</v>
+      </c>
+      <c r="I26" s="14"/>
+      <c r="J26" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="K26" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L26" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M26" s="14" t="s">
         <v>812</v>
       </c>
     </row>
-    <row r="27" ht="40" customHeight="1" spans="1:13">
+    <row r="27" ht="40" customHeight="1" spans="1:12">
       <c r="A27" s="21" t="s">
         <v>68</v>
       </c>
@@ -12936,21 +12870,18 @@
         <v>140</v>
       </c>
       <c r="H27" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I27" s="21" t="s">
-        <v>65</v>
-      </c>
-      <c r="J27" s="4"/>
-      <c r="K27" s="20"/>
+        <v>65</v>
+      </c>
+      <c r="I27" s="4"/>
+      <c r="J27" s="20"/>
+      <c r="K27" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L27" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M27" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="28" ht="40" customHeight="1" spans="1:13">
+    <row r="28" ht="40" customHeight="1" spans="1:12">
       <c r="A28" s="14" t="s">
         <v>59</v>
       </c>
@@ -12973,23 +12904,20 @@
         <v>65</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="I28" s="14" t="s">
         <v>796</v>
       </c>
-      <c r="J28" s="14"/>
+      <c r="I28" s="14"/>
+      <c r="J28" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="K28" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L28" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M28" s="14" t="s">
         <v>819</v>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1" spans="1:13">
+    <row r="29" ht="18" customHeight="1" spans="1:12">
       <c r="A29" s="21" t="s">
         <v>68</v>
       </c>
@@ -13012,21 +12940,18 @@
         <v>140</v>
       </c>
       <c r="H29" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="I29" s="21" t="s">
         <v>796</v>
       </c>
-      <c r="J29" s="4"/>
-      <c r="K29" s="20"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="20"/>
+      <c r="K29" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L29" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M29" s="4" t="s">
         <v>823</v>
       </c>
     </row>
-    <row r="30" ht="30" customHeight="1" spans="1:13">
+    <row r="30" ht="30" customHeight="1" spans="1:12">
       <c r="A30" s="14" t="s">
         <v>59</v>
       </c>
@@ -13049,23 +12974,20 @@
         <v>65</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="I30" s="14" t="s">
         <v>748</v>
       </c>
-      <c r="J30" s="14"/>
+      <c r="I30" s="14"/>
+      <c r="J30" s="14" t="s">
+        <v>65</v>
+      </c>
       <c r="K30" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L30" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M30" s="14" t="s">
         <v>827</v>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" spans="1:13">
+    <row r="31" ht="16.5" customHeight="1" spans="1:12">
       <c r="A31" s="4" t="s">
         <v>68</v>
       </c>
@@ -13088,30 +13010,27 @@
         <v>140</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I31" s="4" t="s">
         <v>758</v>
       </c>
-      <c r="J31" s="4"/>
-      <c r="K31" s="20"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="20"/>
+      <c r="K31" s="4" t="s">
+        <v>65</v>
+      </c>
       <c r="L31" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M31" s="4" t="s">
         <v>831</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A23:M23"/>
-    <mergeCell ref="J6:J8"/>
-    <mergeCell ref="J10:J12"/>
-    <mergeCell ref="J15:J16"/>
-    <mergeCell ref="J18:J22"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A23:L23"/>
+    <mergeCell ref="I6:I8"/>
+    <mergeCell ref="I10:I12"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="I18:I22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
@@ -13125,7 +13044,7 @@
     <tabColor rgb="FFC55A11"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
@@ -13135,25 +13054,24 @@
     <col min="5" max="5" width="7" customWidth="1"/>
     <col min="6" max="6" width="38" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
-    <col min="10" max="10" width="9" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
-    <col min="13" max="13" width="22" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="9" customWidth="1"/>
+    <col min="10" max="10" width="11" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="12" max="12" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customHeight="1" spans="1:13">
+    <row r="1" ht="20.25" customHeight="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>832</v>
       </c>
     </row>
-    <row r="2" ht="40" customHeight="1" spans="1:13">
+    <row r="2" ht="40" customHeight="1" spans="1:12">
       <c r="A2" s="2" t="s">
         <v>833</v>
       </c>
     </row>
-    <row r="3" ht="32" customHeight="1" spans="1:13">
+    <row r="3" ht="32" customHeight="1" spans="1:12">
       <c r="A3" s="3" t="s">
         <v>44</v>
       </c>
@@ -13176,30 +13094,27 @@
         <v>51</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="M3" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" ht="40" customHeight="1" spans="1:13">
+    <row r="4" ht="40" customHeight="1" spans="1:12">
       <c r="A4" s="13" t="s">
         <v>834</v>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1" spans="1:13">
+    <row r="5" ht="40" customHeight="1" spans="1:12">
       <c r="A5" s="14" t="s">
         <v>835</v>
       </c>
@@ -13222,7 +13137,7 @@
         <v>65</v>
       </c>
       <c r="H5" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I5" s="14" t="s">
         <v>65</v>
@@ -13231,16 +13146,13 @@
         <v>65</v>
       </c>
       <c r="K5" s="14" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L5" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="M5" s="14" t="s">
         <v>840</v>
       </c>
     </row>
-    <row r="6" ht="40" customHeight="1" spans="1:13">
+    <row r="6" ht="40" customHeight="1" spans="1:12">
       <c r="A6" s="4" t="s">
         <v>68</v>
       </c>
@@ -13263,25 +13175,18 @@
         <v>73</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="J6" s="4">
-        <v>15</v>
-      </c>
+        <v>65</v>
+      </c>
+      <c r="I6" s="4"/>
+      <c r="J6" s="4"/>
       <c r="K6" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M6" s="4" t="s">
         <v>844</v>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1" spans="1:13">
+    <row r="7" ht="40" customHeight="1" spans="1:12">
       <c r="A7" s="4" t="s">
         <v>68</v>
       </c>
@@ -13304,25 +13209,18 @@
         <v>73</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I7" s="4" t="s">
         <v>841</v>
       </c>
-      <c r="J7" s="4">
-        <v>8</v>
-      </c>
+      <c r="I7" s="4"/>
+      <c r="J7" s="4"/>
       <c r="K7" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M7" s="4" t="s">
         <v>848</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" spans="1:13">
+    <row r="8" ht="18" customHeight="1" spans="1:12">
       <c r="A8" s="4" t="s">
         <v>68</v>
       </c>
@@ -13345,30 +13243,23 @@
         <v>73</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I8" s="4" t="s">
         <v>841</v>
       </c>
-      <c r="J8" s="4">
-        <v>5</v>
-      </c>
+      <c r="I8" s="4"/>
+      <c r="J8" s="4"/>
       <c r="K8" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M8" s="4" t="s">
         <v>852</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" spans="1:13">
+    <row r="9" ht="15.75" customHeight="1" spans="1:12">
       <c r="A9" s="17" t="s">
         <v>853</v>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" spans="1:13">
+    <row r="10" ht="16.5" customHeight="1" spans="1:12">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -13391,25 +13282,18 @@
         <v>140</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I10" s="4" t="s">
         <v>845</v>
       </c>
-      <c r="J10" s="4">
-        <v>13</v>
-      </c>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
       <c r="K10" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L10" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M10" s="4" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" spans="1:13">
+    <row r="11" ht="16.5" customHeight="1" spans="1:12">
       <c r="A11" s="4" t="s">
         <v>68</v>
       </c>
@@ -13432,25 +13316,18 @@
         <v>140</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I11" s="4" t="s">
         <v>845</v>
       </c>
-      <c r="J11" s="4">
-        <v>10</v>
-      </c>
+      <c r="I11" s="4"/>
+      <c r="J11" s="4"/>
       <c r="K11" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L11" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M11" s="4" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" spans="1:13">
+    <row r="12" ht="16.5" customHeight="1" spans="1:12">
       <c r="A12" s="4" t="s">
         <v>68</v>
       </c>
@@ -13473,25 +13350,18 @@
         <v>140</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I12" s="4" t="s">
         <v>845</v>
       </c>
-      <c r="J12" s="4">
-        <v>10</v>
-      </c>
+      <c r="I12" s="4"/>
+      <c r="J12" s="4"/>
       <c r="K12" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L12" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M12" s="4" t="s">
         <v>857</v>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" spans="1:13">
+    <row r="13" ht="16.5" customHeight="1" spans="1:12">
       <c r="A13" s="4" t="s">
         <v>68</v>
       </c>
@@ -13514,30 +13384,23 @@
         <v>140</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="I13" s="4" t="s">
         <v>854</v>
       </c>
-      <c r="J13" s="4">
-        <v>8</v>
-      </c>
+      <c r="I13" s="4"/>
+      <c r="J13" s="4"/>
       <c r="K13" s="4" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="L13" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="M13" s="4" t="s">
         <v>857</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A4:M4"/>
-    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A4:L4"/>
+    <mergeCell ref="A9:L9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" fitToHeight="0" orientation="landscape"/>
@@ -13551,190 +13414,150 @@
     <tabColor rgb="FF548235"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:E10"/>
+  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="16" customWidth="1"/>
     <col min="4" max="4" width="40" customWidth="1"/>
-    <col min="5" max="6" width="28" customWidth="1"/>
+    <col min="5" max="5" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20.25" customHeight="1" spans="1:6">
+    <row r="1" ht="20.25" customHeight="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>866</v>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1" spans="1:6">
-      <c r="A2" s="2" t="s">
+    <row r="2" ht="50" customHeight="1" spans="1:5">
+      <c r="A2" s="2"/>
+    </row>
+    <row r="3" ht="32" customHeight="1" spans="1:5">
+      <c r="A3" s="3" t="s">
         <v>867</v>
       </c>
-    </row>
-    <row r="3" ht="32" customHeight="1" spans="1:6">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="3" t="s">
         <v>868</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>869</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>870</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>871</v>
       </c>
-      <c r="E3" s="3" t="s">
+    </row>
+    <row r="4" ht="120" customHeight="1" spans="1:5">
+      <c r="A4" s="7" t="s">
         <v>872</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="7" t="s">
         <v>873</v>
       </c>
-    </row>
-    <row r="4" ht="120" customHeight="1" spans="1:6">
-      <c r="A4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>874</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>875</v>
       </c>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="5" ht="90" customHeight="1" spans="1:5">
+      <c r="A5" s="7" t="s">
         <v>876</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="B5" s="7"/>
+      <c r="C5" s="7" t="s">
         <v>877</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="D5" s="7" t="s">
         <v>878</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>879</v>
       </c>
     </row>
-    <row r="5" ht="90" customHeight="1" spans="1:6">
-      <c r="A5" s="8" t="s">
+    <row r="6" ht="90" customHeight="1" spans="1:5">
+      <c r="A6" s="7" t="s">
         <v>880</v>
       </c>
-      <c r="B5" s="8" t="s">
+      <c r="B6" s="7"/>
+      <c r="C6" s="9" t="s">
         <v>881</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="D6" s="7" t="s">
         <v>882</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>883</v>
       </c>
-      <c r="E5" s="8" t="s">
+    </row>
+    <row r="7" ht="90" customHeight="1" spans="1:5">
+      <c r="A7" s="8" t="s">
         <v>884</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="B7" s="7"/>
+      <c r="C7" s="7" t="s">
         <v>885</v>
       </c>
-    </row>
-    <row r="6" ht="90" customHeight="1" spans="1:6">
-      <c r="A6" s="8" t="s">
+      <c r="D7" s="7" t="s">
         <v>886</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="E7" s="7" t="s">
         <v>887</v>
       </c>
-      <c r="C6" s="9" t="s">
+    </row>
+    <row r="8" ht="90" customHeight="1" spans="1:5">
+      <c r="A8" s="8" t="s">
         <v>888</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="B8" s="8"/>
+      <c r="C8" s="7" t="s">
         <v>889</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="D8" s="8" t="s">
         <v>890</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="E8" s="7" t="s">
         <v>891</v>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1" spans="1:6">
-      <c r="A7" s="8" t="s">
+    <row r="9" ht="90" customHeight="1" spans="1:5">
+      <c r="A9" s="10" t="s">
         <v>892</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B9" s="11"/>
+      <c r="C9" s="10" t="s">
         <v>893</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="D9" s="10" t="s">
         <v>894</v>
       </c>
-      <c r="D7" s="8" t="s">
+      <c r="E9" s="10" t="s">
         <v>895</v>
       </c>
-      <c r="E7" s="8" t="s">
+    </row>
+    <row r="10" ht="90" customHeight="1" spans="1:5">
+      <c r="A10" s="12" t="s">
         <v>896</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="B10" s="12"/>
+      <c r="C10" s="12" t="s">
         <v>897</v>
       </c>
-    </row>
-    <row r="8" ht="90" customHeight="1" spans="1:6">
-      <c r="A8" s="10" t="s">
+      <c r="D10" s="12" t="s">
         <v>898</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="E10" s="12" t="s">
         <v>899</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>900</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>901</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>902</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="9" ht="90" customHeight="1" spans="1:6">
-      <c r="A9" s="11" t="s">
-        <v>904</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>905</v>
-      </c>
-      <c r="C9" s="11" t="s">
-        <v>906</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>907</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>908</v>
-      </c>
-      <c r="F9" s="11" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="10" ht="90" customHeight="1" spans="1:6">
-      <c r="A10" s="12" t="s">
-        <v>910</v>
-      </c>
-      <c r="B10" s="12" t="s">
-        <v>911</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>912</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>913</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>914</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>915</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="1" orientation="landscape"/>

</xml_diff>

<commit_message>
vault backup: 2026-07-21 14:56:47
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/MVP功能清单.xlsx
+++ b/公司项目/认知行动/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12420" firstSheet="2" activeTab="8"/>
+    <workbookView windowWidth="28800" windowHeight="12420" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="说明" sheetId="1" r:id="rId1"/>
@@ -129,6 +129,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">OCC </t>
     </r>
     <r>
@@ -145,6 +150,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve">DC </t>
     </r>
     <r>
@@ -364,6 +374,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
       <t>真机</t>
     </r>
     <r>
@@ -937,7 +953,7 @@
     <t>R-MC-013</t>
   </si>
   <si>
-    <t>行动关系(agent_id+account_id+terminal_id+proxy_id)读写，单一存储 mc_binding；agent:账号=1:N，账号:终端:IP=1:1:1</t>
+    <t>行动关系</t>
   </si>
   <si>
     <t>agent:account:终端:IP = 1:N:1:1</t>
@@ -1265,12 +1281,6 @@
   </si>
   <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
       <t>【</t>
     </r>
     <r>
@@ -1280,7 +1290,7 @@
         <rFont val="Calibri"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">V1.1 · </t>
+      <t xml:space="preserve">V1.1 </t>
     </r>
     <r>
       <rPr>
@@ -1289,269 +1299,173 @@
         <rFont val="Noto Serif CJK SC"/>
         <charset val="134"/>
       </rPr>
-      <t>后台增强】（第</t>
+      <t>】</t>
     </r>
+  </si>
+  <si>
+    <t>F-MC-01-02</t>
+  </si>
+  <si>
+    <t>浏览器Profile创建与CDP接入</t>
+  </si>
+  <si>
+    <t>V1.2</t>
+  </si>
+  <si>
+    <t>桌面端指纹浏览器Profile接入</t>
+  </si>
+  <si>
+    <t>依赖商用指纹浏览器EI-06</t>
+  </si>
+  <si>
+    <t>F-MC-02-01</t>
+  </si>
+  <si>
+    <t>浏览器Profile指纹固化</t>
+  </si>
+  <si>
+    <t>Profile指纹固化配置</t>
+  </si>
+  <si>
+    <t>指纹浏览器相关</t>
+  </si>
+  <si>
+    <t>F-MC-03-03</t>
+  </si>
+  <si>
+    <t>风控信号识别与规避</t>
+  </si>
+  <si>
+    <t>风控对抗进阶</t>
+  </si>
+  <si>
+    <t>F-MC-03-02</t>
+  </si>
+  <si>
+    <t>F-MC-04-02</t>
+  </si>
+  <si>
+    <t>桌面端商用API画面远控</t>
+  </si>
+  <si>
+    <t>桌面端CDP画面远控</t>
+  </si>
+  <si>
+    <t>F-MC-04-04</t>
+  </si>
+  <si>
+    <t>剪贴板双向同步</t>
+  </si>
+  <si>
+    <t>F-MC-09-04</t>
+  </si>
+  <si>
+    <t>状态变更联动</t>
+  </si>
+  <si>
+    <t>多系统状态联动</t>
+  </si>
+  <si>
+    <t>F-MC-10-06</t>
+  </si>
+  <si>
+    <t>内容触达与互动统计</t>
+  </si>
+  <si>
+    <t>触达/互动统计</t>
+  </si>
+  <si>
+    <t>F-MC-10-07</t>
+  </si>
+  <si>
+    <t>账号健康度统计</t>
+  </si>
+  <si>
+    <t>账号健康度模型</t>
+  </si>
+  <si>
+    <t>F-MC-10-08</t>
+  </si>
+  <si>
+    <t>任务复盘归因</t>
+  </si>
+  <si>
+    <t>复盘归因分析</t>
+  </si>
+  <si>
+    <t>F-MC-11-04</t>
+  </si>
+  <si>
+    <t>账号验证与风险识别</t>
+  </si>
+  <si>
+    <t>账号风险评估/分类</t>
+  </si>
+  <si>
+    <t>M-MC-12</t>
+  </si>
+  <si>
+    <t>智能体账号分层分组</t>
+  </si>
+  <si>
+    <t>R-MC-012</t>
+  </si>
+  <si>
+    <t>账号组织进阶</t>
+  </si>
+  <si>
+    <t>F-MC-12-01</t>
+  </si>
+  <si>
+    <t>分层分组管理</t>
+  </si>
+  <si>
+    <t>F-MC-12-02</t>
+  </si>
+  <si>
+    <t>智能体账号作业生命周期</t>
+  </si>
+  <si>
+    <t>作业生命周期</t>
+  </si>
+  <si>
+    <t>F-MC-13-03</t>
+  </si>
+  <si>
+    <t>账号资产抽取</t>
+  </si>
+  <si>
+    <t>资产抽取</t>
+  </si>
+  <si>
+    <t>F-MC-13-04</t>
+  </si>
+  <si>
+    <t>迁移目标账号校验</t>
+  </si>
+  <si>
+    <t>目标账号校验</t>
+  </si>
+  <si>
+    <t>F-MC-13-05</t>
+  </si>
+  <si>
+    <t>继承写入与绑定切换</t>
+  </si>
+  <si>
+    <t>继承写入/绑定切换</t>
+  </si>
+  <si>
+    <t>F-MC-14-04</t>
+  </si>
+  <si>
+    <t>智能体定义更新生效</t>
+  </si>
+  <si>
+    <t>版本更新生效</t>
+  </si>
+  <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve">5-7 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>月</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> · </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>后</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1+</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>后</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2+</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>前</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>）</t>
-    </r>
-  </si>
-  <si>
-    <t>F-MC-01-02</t>
-  </si>
-  <si>
-    <t>浏览器Profile创建与CDP接入</t>
-  </si>
-  <si>
-    <t>V1.2</t>
-  </si>
-  <si>
-    <t>桌面端指纹浏览器Profile接入</t>
-  </si>
-  <si>
-    <t>依赖商用指纹浏览器EI-06</t>
-  </si>
-  <si>
-    <t>F-MC-02-01</t>
-  </si>
-  <si>
-    <t>浏览器Profile指纹固化</t>
-  </si>
-  <si>
-    <t>Profile指纹固化配置</t>
-  </si>
-  <si>
-    <t>指纹浏览器相关</t>
-  </si>
-  <si>
-    <t>F-MC-03-03</t>
-  </si>
-  <si>
-    <t>风控信号识别与规避</t>
-  </si>
-  <si>
-    <t>风控对抗进阶</t>
-  </si>
-  <si>
-    <t>F-MC-03-02</t>
-  </si>
-  <si>
-    <t>F-MC-04-02</t>
-  </si>
-  <si>
-    <t>桌面端商用API画面远控</t>
-  </si>
-  <si>
-    <t>桌面端CDP画面远控</t>
-  </si>
-  <si>
-    <t>F-MC-04-04</t>
-  </si>
-  <si>
-    <t>剪贴板双向同步</t>
-  </si>
-  <si>
-    <t>F-MC-09-04</t>
-  </si>
-  <si>
-    <t>状态变更联动</t>
-  </si>
-  <si>
-    <t>多系统状态联动</t>
-  </si>
-  <si>
-    <t>F-MC-10-06</t>
-  </si>
-  <si>
-    <t>内容触达与互动统计</t>
-  </si>
-  <si>
-    <t>触达/互动统计</t>
-  </si>
-  <si>
-    <t>F-MC-10-07</t>
-  </si>
-  <si>
-    <t>账号健康度统计</t>
-  </si>
-  <si>
-    <t>账号健康度模型</t>
-  </si>
-  <si>
-    <t>F-MC-10-08</t>
-  </si>
-  <si>
-    <t>任务复盘归因</t>
-  </si>
-  <si>
-    <t>复盘归因分析</t>
-  </si>
-  <si>
-    <t>F-MC-11-04</t>
-  </si>
-  <si>
-    <t>账号验证与风险识别</t>
-  </si>
-  <si>
-    <t>账号风险评估/分类</t>
-  </si>
-  <si>
-    <t>M-MC-12</t>
-  </si>
-  <si>
-    <t>智能体账号分层分组</t>
-  </si>
-  <si>
-    <t>R-MC-012</t>
-  </si>
-  <si>
-    <t>账号组织进阶</t>
-  </si>
-  <si>
-    <t>F-MC-12-01</t>
-  </si>
-  <si>
-    <t>分层分组管理</t>
-  </si>
-  <si>
-    <t>F-MC-12-02</t>
-  </si>
-  <si>
-    <t>智能体账号作业生命周期</t>
-  </si>
-  <si>
-    <t>作业生命周期</t>
-  </si>
-  <si>
-    <t>F-MC-13-03</t>
-  </si>
-  <si>
-    <t>账号资产抽取</t>
-  </si>
-  <si>
-    <t>资产抽取</t>
-  </si>
-  <si>
-    <t>F-MC-13-04</t>
-  </si>
-  <si>
-    <t>迁移目标账号校验</t>
-  </si>
-  <si>
-    <t>目标账号校验</t>
-  </si>
-  <si>
-    <t>F-MC-13-05</t>
-  </si>
-  <si>
-    <t>继承写入与绑定切换</t>
-  </si>
-  <si>
-    <t>继承写入/绑定切换</t>
-  </si>
-  <si>
-    <t>F-MC-14-04</t>
-  </si>
-  <si>
-    <t>智能体定义更新生效</t>
-  </si>
-  <si>
-    <t>版本更新生效</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
       <t>【</t>
     </r>
     <r>
@@ -1570,79 +1484,7 @@
         <rFont val="Noto Serif CJK SC"/>
         <charset val="134"/>
       </rPr>
-      <t>深化】（第</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> 7-8 </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>月</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t xml:space="preserve"> · </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>后</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>1+</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>后</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <charset val="134"/>
-      </rPr>
-      <t>2</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <rFont val="Noto Serif CJK SC"/>
-        <charset val="134"/>
-      </rPr>
-      <t>）</t>
+      <t>深化】</t>
     </r>
   </si>
   <si>
@@ -2077,6 +1919,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF595959"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t xml:space="preserve"> </t>
     </r>
     <r>
@@ -3227,6 +3075,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>M1</t>
     </r>
     <r>
@@ -3257,6 +3110,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>M2</t>
     </r>
     <r>
@@ -3277,6 +3136,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
       <t>第</t>
     </r>
     <r>
@@ -3314,6 +3178,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>M3</t>
     </r>
     <r>
@@ -3330,6 +3199,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>OCC</t>
     </r>
     <r>
@@ -3375,6 +3249,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Noto Serif CJK SC"/>
+        <charset val="134"/>
+      </rPr>
       <t>第</t>
     </r>
     <r>
@@ -3396,6 +3275,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>M4</t>
     </r>
     <r>
@@ -3412,6 +3296,11 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Calibri"/>
+        <charset val="134"/>
+      </rPr>
       <t>OCC</t>
     </r>
     <r>
@@ -3575,7 +3464,7 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="47">
+  <fonts count="51">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3652,6 +3541,11 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="14"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="18"/>
       <color rgb="FFFF0000"/>
       <name val="Noto Serif CJK SC"/>
@@ -3659,9 +3553,15 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color rgb="FFFFFFFF"/>
       <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3671,8 +3571,19 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="14"/>
+      <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
+      <name val="Noto Serif CJK SC"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
@@ -3869,15 +3780,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="22"/>
-      <color rgb="FFFF0000"/>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF1F4E79"/>
       <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="18"/>
+      <sz val="22"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Noto Serif CJK SC"/>
       <charset val="134"/>
     </font>
     <font>
@@ -3888,10 +3800,9 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="16"/>
-      <color rgb="FF1F4E79"/>
-      <name val="Noto Serif CJK SC"/>
+      <sz val="18"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -4234,152 +4145,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="43" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="44" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="9" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="23" fillId="0" borderId="0">
+    <xf numFmtId="41" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="23" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0">
+    <xf numFmtId="42" fontId="27" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2">
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="3">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="31" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="4">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="12" borderId="5">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="12" borderId="4">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="2">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="13" borderId="6">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="3">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="8">
+    <xf numFmtId="0" fontId="36" fillId="11" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="37" fillId="12" borderId="5">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="3" borderId="0">
+    <xf numFmtId="0" fontId="38" fillId="12" borderId="4">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="4" borderId="0">
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="6">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="15" borderId="0">
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="8">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="17" borderId="0">
+    <xf numFmtId="0" fontId="42" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="43" fillId="3" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="19" borderId="0">
+    <xf numFmtId="0" fontId="44" fillId="4" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="21" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="23" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="25" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="27" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="29" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="31" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="33" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="35" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="36" borderId="0">
+    <xf numFmtId="0" fontId="45" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="42" fillId="37" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="41" fillId="38" borderId="0">
+    <xf numFmtId="0" fontId="46" fillId="33" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="38" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4459,24 +4370,42 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -4485,13 +4414,19 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4504,13 +4439,13 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -4917,65 +4852,65 @@
   </cols>
   <sheetData>
     <row r="1" ht="23.25" customHeight="1" spans="1:2">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:2">
-      <c r="A3" s="40" t="s">
+      <c r="A3" s="48" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="48" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:2">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="42" t="s">
+      <c r="B4" s="50" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:2">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="42" t="s">
+      <c r="B5" s="50" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:2">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="49" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="50" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:2">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="49" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="43">
+      <c r="B7" s="51">
         <v>46223</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:2">
-      <c r="A8" s="42" t="s">
+      <c r="A8" s="50" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="42" t="s">
+      <c r="B8" s="50" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:2">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="52" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="10" ht="55" customHeight="1" spans="1:2">
-      <c r="A10" s="42" t="s">
+      <c r="A10" s="50" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4985,17 +4920,17 @@
       </c>
     </row>
     <row r="12" ht="55" customHeight="1" spans="1:2">
-      <c r="A12" s="42" t="s">
+      <c r="A12" s="50" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="1:2">
-      <c r="A13" s="45" t="s">
+      <c r="A13" s="53" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="14" ht="55" customHeight="1" spans="1:2">
-      <c r="A14" s="42" t="s">
+      <c r="A14" s="50" t="s">
         <v>16</v>
       </c>
     </row>
@@ -5005,20 +4940,20 @@
       </c>
     </row>
     <row r="16" ht="25" customHeight="1" spans="1:2">
-      <c r="A16" s="46" t="s">
+      <c r="A16" s="54" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1" spans="1:3">
-      <c r="A17" s="44" t="s">
+      <c r="A17" s="52" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:3">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="47"/>
+      <c r="C18" s="55"/>
     </row>
     <row r="19" ht="22" customHeight="1" spans="1:3">
       <c r="A19" s="24" t="s">
@@ -5026,34 +4961,34 @@
       </c>
     </row>
     <row r="20" ht="22" customHeight="1" spans="1:3">
-      <c r="A20" s="42" t="s">
+      <c r="A20" s="50" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="42" t="s">
+      <c r="B20" s="50" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1" spans="1:3">
-      <c r="A21" s="42" t="s">
+      <c r="A21" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="42" t="s">
+      <c r="B21" s="50" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1" spans="1:3">
-      <c r="A22" s="42" t="s">
+      <c r="A22" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="42" t="s">
+      <c r="B22" s="50" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1" spans="1:3">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="50" t="s">
         <v>28</v>
       </c>
-      <c r="B23" s="42" t="s">
+      <c r="B23" s="50" t="s">
         <v>29</v>
       </c>
       <c r="C23">
@@ -5061,10 +4996,10 @@
       </c>
     </row>
     <row r="24" ht="22" customHeight="1" spans="1:3">
-      <c r="A24" s="48" t="s">
+      <c r="A24" s="56" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="42" t="s">
+      <c r="B24" s="50" t="s">
         <v>31</v>
       </c>
       <c r="C24">
@@ -5072,10 +5007,10 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1" spans="1:3">
-      <c r="A25" s="48" t="s">
+      <c r="A25" s="56" t="s">
         <v>32</v>
       </c>
-      <c r="B25" s="42" t="s">
+      <c r="B25" s="50" t="s">
         <v>33</v>
       </c>
       <c r="C25">
@@ -5083,10 +5018,10 @@
       </c>
     </row>
     <row r="26" ht="22" customHeight="1" spans="1:3">
-      <c r="A26" s="42" t="s">
+      <c r="A26" s="50" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="42" t="s">
+      <c r="B26" s="50" t="s">
         <v>35</v>
       </c>
       <c r="C26">
@@ -5094,10 +5029,10 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1" spans="1:3">
-      <c r="A27" s="42" t="s">
+      <c r="A27" s="50" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="42" t="s">
+      <c r="B27" s="50" t="s">
         <v>37</v>
       </c>
       <c r="C27">
@@ -5105,10 +5040,10 @@
       </c>
     </row>
     <row r="28" ht="22" customHeight="1" spans="1:3">
-      <c r="A28" s="42" t="s">
+      <c r="A28" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="B28" s="42" t="s">
+      <c r="B28" s="50" t="s">
         <v>39</v>
       </c>
       <c r="C28">
@@ -5116,10 +5051,10 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:3">
-      <c r="A29" s="42" t="s">
+      <c r="A29" s="50" t="s">
         <v>40</v>
       </c>
-      <c r="B29" s="42" t="s">
+      <c r="B29" s="50" t="s">
         <v>41</v>
       </c>
     </row>
@@ -5287,10 +5222,11 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N84"/>
-  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="7.2" defaultRowHeight="18"/>
   <cols>
     <col min="1" max="1" width="7" customWidth="1"/>
-    <col min="2" max="3" width="14" customWidth="1"/>
+    <col min="2" max="2" width="14" style="28" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="7" customWidth="1"/>
@@ -5310,7 +5246,7 @@
       </c>
     </row>
     <row r="2" ht="40" customHeight="1" spans="1:14">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="29" t="s">
         <v>43</v>
       </c>
     </row>
@@ -5318,7 +5254,7 @@
       <c r="A3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>45</v>
       </c>
       <c r="C3" s="3" t="s">
@@ -5367,11 +5303,11 @@
       <c r="A5" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="14"/>
+      <c r="B5" s="31"/>
       <c r="C5" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="32" t="s">
         <v>61</v>
       </c>
       <c r="E5" s="14" t="s">
@@ -5409,7 +5345,7 @@
       <c r="A6" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="33" t="s">
         <v>69</v>
       </c>
       <c r="C6" s="4" t="s">
@@ -5453,7 +5389,7 @@
       <c r="A7" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="16"/>
+      <c r="B7" s="34"/>
       <c r="C7" s="4" t="s">
         <v>76</v>
       </c>
@@ -5493,7 +5429,7 @@
       <c r="A8" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B8" s="16"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="4" t="s">
         <v>79</v>
       </c>
@@ -5533,7 +5469,7 @@
       <c r="A9" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B9" s="16"/>
+      <c r="B9" s="34"/>
       <c r="C9" s="4" t="s">
         <v>84</v>
       </c>
@@ -5573,7 +5509,7 @@
       <c r="A10" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B10" s="16"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="4" t="s">
         <v>88</v>
       </c>
@@ -5611,11 +5547,11 @@
       <c r="A11" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="31"/>
       <c r="C11" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="D11" s="30" t="s">
+      <c r="D11" s="32" t="s">
         <v>93</v>
       </c>
       <c r="E11" s="14" t="s">
@@ -5651,7 +5587,7 @@
       <c r="A12" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="31" t="s">
+      <c r="B12" s="33" t="s">
         <v>97</v>
       </c>
       <c r="C12" t="s">
@@ -5692,7 +5628,7 @@
       <c r="A13" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="32"/>
+      <c r="B13" s="35"/>
       <c r="C13" t="s">
         <v>103</v>
       </c>
@@ -5732,7 +5668,7 @@
       <c r="A14" t="s">
         <v>68</v>
       </c>
-      <c r="B14" s="32"/>
+      <c r="B14" s="35"/>
       <c r="C14" t="s">
         <v>108</v>
       </c>
@@ -5769,7 +5705,7 @@
       <c r="A15" t="s">
         <v>68</v>
       </c>
-      <c r="B15" s="32"/>
+      <c r="B15" s="35"/>
       <c r="C15" t="s">
         <v>112</v>
       </c>
@@ -5806,7 +5742,7 @@
       <c r="A16" t="s">
         <v>68</v>
       </c>
-      <c r="B16" s="32"/>
+      <c r="B16" s="35"/>
       <c r="C16" t="s">
         <v>116</v>
       </c>
@@ -5843,7 +5779,7 @@
       <c r="A17" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="32"/>
+      <c r="B17" s="35"/>
       <c r="C17" t="s">
         <v>120</v>
       </c>
@@ -5883,7 +5819,7 @@
       <c r="A18" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="31"/>
       <c r="C18" s="14" t="s">
         <v>125</v>
       </c>
@@ -5925,7 +5861,7 @@
       <c r="A19" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C19" s="4" t="s">
@@ -5969,7 +5905,7 @@
       <c r="A20" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B20" s="16"/>
+      <c r="B20" s="34"/>
       <c r="C20" s="4" t="s">
         <v>137</v>
       </c>
@@ -6009,7 +5945,7 @@
       <c r="A21" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="16"/>
+      <c r="B21" s="34"/>
       <c r="C21" s="21" t="s">
         <v>142</v>
       </c>
@@ -6049,7 +5985,7 @@
       <c r="A22" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="34"/>
       <c r="C22" s="21" t="s">
         <v>147</v>
       </c>
@@ -6089,7 +6025,7 @@
       <c r="A23" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B23" s="16"/>
+      <c r="B23" s="34"/>
       <c r="C23" s="4" t="s">
         <v>152</v>
       </c>
@@ -6129,7 +6065,7 @@
       <c r="A24" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B24" s="16"/>
+      <c r="B24" s="34"/>
       <c r="C24" s="4" t="s">
         <v>158</v>
       </c>
@@ -6169,7 +6105,7 @@
       <c r="A25" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="14" t="s">
         <v>161</v>
       </c>
@@ -6211,7 +6147,7 @@
       <c r="A26" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B26" s="16" t="s">
+      <c r="B26" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C26" s="4" t="s">
@@ -6255,7 +6191,7 @@
       <c r="A27" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="16"/>
+      <c r="B27" s="34"/>
       <c r="C27" s="4" t="s">
         <v>170</v>
       </c>
@@ -6274,7 +6210,7 @@
       <c r="H27" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="I27" s="33" t="s">
+      <c r="I27" s="36" t="s">
         <v>66</v>
       </c>
       <c r="J27" s="4" t="s">
@@ -6295,7 +6231,7 @@
       <c r="A28" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="14"/>
+      <c r="B28" s="31"/>
       <c r="C28" s="14" t="s">
         <v>176</v>
       </c>
@@ -6337,7 +6273,7 @@
       <c r="A29" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B29" s="27" t="s">
+      <c r="B29" s="33" t="s">
         <v>97</v>
       </c>
       <c r="C29" s="4" t="s">
@@ -6381,7 +6317,7 @@
       <c r="A30" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="4" t="s">
         <v>186</v>
       </c>
@@ -6421,7 +6357,7 @@
       <c r="A31" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B31" s="14"/>
+      <c r="B31" s="31"/>
       <c r="C31" s="14" t="s">
         <v>191</v>
       </c>
@@ -6463,7 +6399,7 @@
       <c r="A32" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C32" s="4" t="s">
@@ -6507,7 +6443,7 @@
       <c r="A33" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B33" s="16"/>
+      <c r="B33" s="34"/>
       <c r="C33" s="4" t="s">
         <v>201</v>
       </c>
@@ -6547,7 +6483,7 @@
       <c r="A34" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="14"/>
+      <c r="B34" s="31"/>
       <c r="C34" s="14" t="s">
         <v>206</v>
       </c>
@@ -6589,7 +6525,7 @@
       <c r="A35" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="16" t="s">
+      <c r="B35" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C35" s="4" t="s">
@@ -6633,7 +6569,7 @@
       <c r="A36" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B36" s="16"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="4" t="s">
         <v>216</v>
       </c>
@@ -6673,7 +6609,7 @@
       <c r="A37" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B37" s="16"/>
+      <c r="B37" s="34"/>
       <c r="C37" s="21" t="s">
         <v>220</v>
       </c>
@@ -6709,11 +6645,11 @@
         <v>223</v>
       </c>
     </row>
-    <row r="38" ht="93" customHeight="1" spans="1:14">
+    <row r="38" ht="54" customHeight="1" spans="1:14">
       <c r="A38" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B38" s="14"/>
+      <c r="B38" s="31"/>
       <c r="C38" s="14" t="s">
         <v>224</v>
       </c>
@@ -6726,7 +6662,7 @@
       <c r="F38" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="G38" s="15" t="s">
+      <c r="G38" s="37" t="s">
         <v>227</v>
       </c>
       <c r="H38" s="15" t="s">
@@ -6755,7 +6691,7 @@
       <c r="A39" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B39" s="27" t="s">
+      <c r="B39" s="33" t="s">
         <v>229</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -6799,7 +6735,7 @@
       <c r="A40" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B40" s="16"/>
+      <c r="B40" s="34"/>
       <c r="C40" s="4" t="s">
         <v>234</v>
       </c>
@@ -6839,7 +6775,7 @@
       <c r="A41" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B41" s="14"/>
+      <c r="B41" s="31"/>
       <c r="C41" s="14" t="s">
         <v>238</v>
       </c>
@@ -6881,7 +6817,7 @@
       <c r="A42" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B42" s="16" t="s">
+      <c r="B42" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C42" s="4" t="s">
@@ -6925,7 +6861,7 @@
       <c r="A43" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B43" s="16"/>
+      <c r="B43" s="34"/>
       <c r="C43" s="4" t="s">
         <v>247</v>
       </c>
@@ -6965,7 +6901,7 @@
       <c r="A44" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B44" s="16"/>
+      <c r="B44" s="34"/>
       <c r="C44" s="21" t="s">
         <v>250</v>
       </c>
@@ -7005,7 +6941,7 @@
       <c r="A45" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B45" s="16"/>
+      <c r="B45" s="34"/>
       <c r="C45" s="4" t="s">
         <v>254</v>
       </c>
@@ -7045,7 +6981,7 @@
       <c r="A46" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="14"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="14" t="s">
         <v>257</v>
       </c>
@@ -7087,7 +7023,7 @@
       <c r="A47" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B47" s="27" t="s">
+      <c r="B47" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C47" s="4" t="s">
@@ -7131,7 +7067,7 @@
       <c r="A48" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B48" s="16"/>
+      <c r="B48" s="34"/>
       <c r="C48" s="4" t="s">
         <v>265</v>
       </c>
@@ -7171,7 +7107,7 @@
       <c r="A49" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B49" s="16"/>
+      <c r="B49" s="34"/>
       <c r="C49" s="4" t="s">
         <v>268</v>
       </c>
@@ -7211,7 +7147,7 @@
       <c r="A50" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B50" s="16"/>
+      <c r="B50" s="34"/>
       <c r="C50" s="21" t="s">
         <v>271</v>
       </c>
@@ -7251,7 +7187,7 @@
       <c r="A51" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B51" s="16"/>
+      <c r="B51" s="34"/>
       <c r="C51" s="4" t="s">
         <v>275</v>
       </c>
@@ -7291,7 +7227,7 @@
       <c r="A52" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B52" s="14"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="14" t="s">
         <v>279</v>
       </c>
@@ -7333,7 +7269,7 @@
       <c r="A53" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B53" s="22" t="s">
+      <c r="B53" s="38" t="s">
         <v>229</v>
       </c>
       <c r="C53" s="21" t="s">
@@ -7377,7 +7313,7 @@
       <c r="A54" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B54" s="22"/>
+      <c r="B54" s="39"/>
       <c r="C54" s="4" t="s">
         <v>289</v>
       </c>
@@ -7417,7 +7353,7 @@
       <c r="A55" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B55" s="22"/>
+      <c r="B55" s="39"/>
       <c r="C55" s="4" t="s">
         <v>293</v>
       </c>
@@ -7457,7 +7393,7 @@
       <c r="A56" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B56" s="22"/>
+      <c r="B56" s="39"/>
       <c r="C56" s="4" t="s">
         <v>297</v>
       </c>
@@ -7497,7 +7433,7 @@
       <c r="A57" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B57" s="22"/>
+      <c r="B57" s="39"/>
       <c r="C57" s="4" t="s">
         <v>301</v>
       </c>
@@ -7537,7 +7473,7 @@
       <c r="A58" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B58" s="14"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="14" t="s">
         <v>306</v>
       </c>
@@ -7547,7 +7483,7 @@
       <c r="E58" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="F58" s="34" t="s">
+      <c r="F58" s="40" t="s">
         <v>172</v>
       </c>
       <c r="G58" s="15" t="s">
@@ -7579,7 +7515,7 @@
       <c r="A59" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B59" s="16" t="s">
+      <c r="B59" s="33" t="s">
         <v>130</v>
       </c>
       <c r="C59" s="4" t="s">
@@ -7606,7 +7542,7 @@
       <c r="J59" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="K59" s="35" t="s">
+      <c r="K59" s="41" t="s">
         <v>314</v>
       </c>
       <c r="L59" s="20"/>
@@ -7621,7 +7557,7 @@
       <c r="A60" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B60" s="16"/>
+      <c r="B60" s="34"/>
       <c r="C60" s="21" t="s">
         <v>317</v>
       </c>
@@ -7634,7 +7570,7 @@
       <c r="F60" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="G60" s="36" t="s">
+      <c r="G60" s="42" t="s">
         <v>319</v>
       </c>
       <c r="H60" s="22" t="s">
@@ -7659,7 +7595,7 @@
       <c r="A61" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B61" s="16"/>
+      <c r="B61" s="34"/>
       <c r="C61" s="4" t="s">
         <v>322</v>
       </c>
@@ -7697,7 +7633,7 @@
       <c r="A62" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B62" s="16"/>
+      <c r="B62" s="34"/>
       <c r="C62" s="4" t="s">
         <v>326</v>
       </c>
@@ -7735,7 +7671,7 @@
       <c r="A63" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B63" s="16"/>
+      <c r="B63" s="34"/>
       <c r="C63" s="4" t="s">
         <v>330</v>
       </c>
@@ -7773,7 +7709,7 @@
       <c r="A64" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="16"/>
+      <c r="B64" s="34"/>
       <c r="C64" s="4" t="s">
         <v>333</v>
       </c>
@@ -7808,7 +7744,7 @@
       </c>
     </row>
     <row r="65" ht="40" customHeight="1" spans="1:14">
-      <c r="A65" s="37" t="s">
+      <c r="A65" s="43" t="s">
         <v>336</v>
       </c>
     </row>
@@ -7816,7 +7752,7 @@
       <c r="A66" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B66" s="4"/>
+      <c r="B66" s="44"/>
       <c r="C66" s="4" t="s">
         <v>337</v>
       </c>
@@ -7854,7 +7790,7 @@
       <c r="A67" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B67" s="4"/>
+      <c r="B67" s="44"/>
       <c r="C67" s="4" t="s">
         <v>342</v>
       </c>
@@ -7892,7 +7828,7 @@
       <c r="A68" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B68" s="4"/>
+      <c r="B68" s="44"/>
       <c r="C68" s="4" t="s">
         <v>346</v>
       </c>
@@ -7930,7 +7866,7 @@
       <c r="A69" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B69" s="4"/>
+      <c r="B69" s="44"/>
       <c r="C69" s="4" t="s">
         <v>350</v>
       </c>
@@ -7968,7 +7904,7 @@
       <c r="A70" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B70" s="4"/>
+      <c r="B70" s="44"/>
       <c r="C70" s="4" t="s">
         <v>353</v>
       </c>
@@ -8006,7 +7942,7 @@
       <c r="A71" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B71" s="4"/>
+      <c r="B71" s="44"/>
       <c r="C71" s="4" t="s">
         <v>355</v>
       </c>
@@ -8044,7 +7980,7 @@
       <c r="A72" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B72" s="4"/>
+      <c r="B72" s="44"/>
       <c r="C72" s="4" t="s">
         <v>358</v>
       </c>
@@ -8082,7 +8018,7 @@
       <c r="A73" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B73" s="4"/>
+      <c r="B73" s="44"/>
       <c r="C73" s="4" t="s">
         <v>361</v>
       </c>
@@ -8120,7 +8056,7 @@
       <c r="A74" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B74" s="21"/>
+      <c r="B74" s="45"/>
       <c r="C74" s="21" t="s">
         <v>364</v>
       </c>
@@ -8158,7 +8094,7 @@
       <c r="A75" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B75" s="4"/>
+      <c r="B75" s="44"/>
       <c r="C75" s="4" t="s">
         <v>367</v>
       </c>
@@ -8196,7 +8132,7 @@
       <c r="A76" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="B76" s="14"/>
+      <c r="B76" s="31"/>
       <c r="C76" s="14" t="s">
         <v>370</v>
       </c>
@@ -8236,7 +8172,7 @@
       <c r="A77" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B77" s="4"/>
+      <c r="B77" s="44"/>
       <c r="C77" s="4" t="s">
         <v>374</v>
       </c>
@@ -8274,7 +8210,7 @@
       <c r="A78" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B78" s="4"/>
+      <c r="B78" s="44"/>
       <c r="C78" s="4" t="s">
         <v>376</v>
       </c>
@@ -8308,11 +8244,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" ht="18" customHeight="1" spans="1:14">
+    <row r="79" customHeight="1" spans="1:14">
       <c r="A79" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B79" s="4"/>
+      <c r="B79" s="44"/>
       <c r="C79" s="4" t="s">
         <v>379</v>
       </c>
@@ -8350,7 +8286,7 @@
       <c r="A80" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B80" s="4"/>
+      <c r="B80" s="44"/>
       <c r="C80" s="4" t="s">
         <v>382</v>
       </c>
@@ -8388,7 +8324,7 @@
       <c r="A81" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B81" s="4"/>
+      <c r="B81" s="44"/>
       <c r="C81" s="4" t="s">
         <v>385</v>
       </c>
@@ -8426,7 +8362,7 @@
       <c r="A82" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B82" s="4"/>
+      <c r="B82" s="44"/>
       <c r="C82" s="4" t="s">
         <v>388</v>
       </c>
@@ -8461,7 +8397,7 @@
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1" spans="1:14">
-      <c r="A83" s="38" t="s">
+      <c r="A83" s="46" t="s">
         <v>391</v>
       </c>
     </row>
@@ -8469,7 +8405,7 @@
       <c r="A84" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="B84" s="4"/>
+      <c r="B84" s="44"/>
       <c r="C84" s="4" t="s">
         <v>392</v>
       </c>

</xml_diff>

<commit_message>
vault backup: 2026-07-23 13:56:12
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/MVP功能清单.xlsx
+++ b/公司项目/认知行动/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12420"/>
+    <workbookView windowWidth="28800" windowHeight="12420" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="MC 多设备矩阵自动化群控子系统" sheetId="1" r:id="rId1"/>
@@ -3960,7 +3960,7 @@
         <v>29</v>
       </c>
       <c r="K7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L7" s="11" t="s">
         <v>33</v>
@@ -4001,7 +4001,7 @@
         <v>29</v>
       </c>
       <c r="K8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>33</v>
@@ -4124,7 +4124,7 @@
         <v>29</v>
       </c>
       <c r="K11">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L11" t="s">
         <v>56</v>
@@ -4241,7 +4241,7 @@
         <v>53</v>
       </c>
       <c r="K14">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L14" t="s">
         <v>56</v>
@@ -4279,7 +4279,7 @@
         <v>53</v>
       </c>
       <c r="K15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L15" t="s">
         <v>56</v>
@@ -4317,7 +4317,7 @@
         <v>63</v>
       </c>
       <c r="K16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L16" t="s">
         <v>56</v>
@@ -4444,7 +4444,7 @@
         <v>86</v>
       </c>
       <c r="K19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L19" s="11" t="s">
         <v>90</v>
@@ -4567,7 +4567,7 @@
         <v>111</v>
       </c>
       <c r="K22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" s="11" t="s">
         <v>90</v>
@@ -4608,7 +4608,7 @@
         <v>107</v>
       </c>
       <c r="K23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L23" s="11" t="s">
         <v>90</v>
@@ -4821,7 +4821,7 @@
         <v>86</v>
       </c>
       <c r="K28">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L28" t="s">
         <v>56</v>
@@ -4862,7 +4862,7 @@
         <v>137</v>
       </c>
       <c r="K29">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L29" t="s">
         <v>56</v>
@@ -4989,7 +4989,7 @@
         <v>29</v>
       </c>
       <c r="K32">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L32" s="11" t="s">
         <v>33</v>
@@ -5075,7 +5075,7 @@
         <v>23</v>
       </c>
       <c r="K34">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L34" s="11" t="s">
         <v>90</v>
@@ -5243,7 +5243,7 @@
         <v>107</v>
       </c>
       <c r="K38">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L38" s="11" t="s">
         <v>188</v>
@@ -5370,7 +5370,7 @@
         <v>29</v>
       </c>
       <c r="K41">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L41" s="11" t="s">
         <v>33</v>
@@ -5411,7 +5411,7 @@
         <v>199</v>
       </c>
       <c r="K42">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L42" s="11" t="s">
         <v>33</v>
@@ -5452,7 +5452,7 @@
         <v>199</v>
       </c>
       <c r="K43">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L43" s="11" t="s">
         <v>33</v>
@@ -5579,7 +5579,7 @@
         <v>38</v>
       </c>
       <c r="K46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L46" s="11" t="s">
         <v>90</v>
@@ -5620,7 +5620,7 @@
         <v>218</v>
       </c>
       <c r="K47">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L47" s="11" t="s">
         <v>90</v>
@@ -5702,7 +5702,7 @@
         <v>218</v>
       </c>
       <c r="K49">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L49" s="11" t="s">
         <v>90</v>
@@ -5743,7 +5743,7 @@
         <v>221</v>
       </c>
       <c r="K50">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L50" s="11" t="s">
         <v>90</v>
@@ -5993,7 +5993,7 @@
         <v>218</v>
       </c>
       <c r="K56">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L56" s="11" t="s">
         <v>188</v>
@@ -10673,7 +10673,7 @@
         <v>686</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="11" t="s">
         <v>689</v>
@@ -10711,7 +10711,7 @@
         <v>686</v>
       </c>
       <c r="I8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="11" t="s">
         <v>689</v>
@@ -10787,7 +10787,7 @@
         <v>253</v>
       </c>
       <c r="I10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J10" s="11" t="s">
         <v>689</v>
@@ -10825,7 +10825,7 @@
         <v>704</v>
       </c>
       <c r="I11">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J11" s="11" t="s">
         <v>689</v>
@@ -10901,7 +10901,7 @@
         <v>686</v>
       </c>
       <c r="I13">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="11" t="s">
         <v>689</v>
@@ -11015,7 +11015,7 @@
         <v>726</v>
       </c>
       <c r="I16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J16" s="11" t="s">
         <v>689</v>

</xml_diff>

<commit_message>
vault backup: 2026-07-24 09:51:33
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/MVP功能清单.xlsx
+++ b/公司项目/认知行动/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12420" activeTab="5"/>
+    <workbookView windowWidth="28800" windowHeight="12420" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MC 多设备矩阵自动化群控子系统" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2332" uniqueCount="824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2322" uniqueCount="824">
   <si>
     <t>MC 多设备矩阵自动化群控子系统 · 功能清单（V1.0~V1.3）</t>
   </si>
@@ -104,12 +104,12 @@
     <t>收口鉴权/记录/基础熔断；所有真机动作经网关落地</t>
   </si>
   <si>
+    <t>后端模块</t>
+  </si>
+  <si>
     <t>—</t>
   </si>
   <si>
-    <t>后端模块</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
@@ -173,135 +173,135 @@
     <t>失败计数熔断</t>
   </si>
   <si>
+    <t>M-MC-15</t>
+  </si>
+  <si>
+    <t>真机Agent运行时与编排(AI可用)</t>
+  </si>
+  <si>
+    <t>R-MC-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      </t>
+  </si>
+  <si>
+    <t>CON-15 Agent 独立部署单元；借鉴 SonicCloudOrg(已archived,Apache2.0)；真机=Android 3-8台</t>
+  </si>
+  <si>
+    <t>分布式真机控制服务</t>
+  </si>
+  <si>
+    <t>F-MC-15-01</t>
+  </si>
+  <si>
+    <t>Agent注册与鉴权握手</t>
+  </si>
+  <si>
+    <t>Agent 启动经 II-02 WS 连中心侧编排器，agentKey 配置文件校验 + 版本/能力上报(auth消息)；中心侧回 authResult 分配 agentId</t>
+  </si>
+  <si>
+    <t>杨志</t>
+  </si>
+  <si>
+    <t>agentKey 配置文件读，不做密钥轮换</t>
+  </si>
+  <si>
+    <t>F-MC-15-02</t>
+  </si>
+  <si>
+    <t>心跳保活与在线状态判定</t>
+  </si>
+  <si>
+    <t>Agent 周期发 heartBeat(默认30s)，超时(默认90s)判掉线；推 terminal_offline 事件给 M-MC-01 更新台账在线状态</t>
+  </si>
+  <si>
+    <t>MC-02</t>
+  </si>
+  <si>
+    <t>台账在线状态数据源</t>
+  </si>
+  <si>
+    <t>F-MC-15-03</t>
+  </si>
+  <si>
+    <t>设备占用锁</t>
+  </si>
+  <si>
+    <t>设备占用锁(occupy/release)，一台设备同时只让一个会话用(远控/自动化互斥)；内存锁(单 mc-service 副本)，不做分布式锁</t>
+  </si>
+  <si>
+    <t>防远控和自动化并发打架；分布式锁留 V1.2</t>
+  </si>
+  <si>
+    <t>F-MC-15-04</t>
+  </si>
+  <si>
+    <t>ADB控制通道</t>
+  </si>
+  <si>
+    <t>ddmlib 实现 ADB 通道：install/uninstall/pressKey/reboot/screenshot；动作子集(不做交互式 shell 终端)；经 runAction 消息收口(与 F-MC-15-05 共享)</t>
+  </si>
+  <si>
+    <t>Sonic AndroidDeviceBridgeTool 对应</t>
+  </si>
+  <si>
+    <t>F-MC-15-05</t>
+  </si>
+  <si>
+    <t>无障碍控制通道(uia2)</t>
+  </si>
+  <si>
+    <t>引 sonic-driver-core(Maven jar) 封装 uiautomator2-server：UI 元素 find/click/sendKeys/swipe；断言类步骤全砍；经 runAction 消息收口</t>
+  </si>
+  <si>
+    <t>依赖 archived 库 sonic-driver-core；uia2 协议本身稳定</t>
+  </si>
+  <si>
+    <t>F-MC-15-06</t>
+  </si>
+  <si>
+    <t>远控画面源(scrcpy)</t>
+  </si>
+  <si>
+    <t>抄 Sonic ScrcpyInputSocketThread/OutputSocketThread(Apache2.0)；启动 scrcpy server 抓 H.264 → 经 startScrcpy 推到 mc-sfu 指定端口；本功能只产画面源，WebRTC 转发由 M-MC-04 mc-sfu 承担</t>
+  </si>
+  <si>
+    <t>MC-17</t>
+  </si>
+  <si>
+    <t>媒体面 Agent→mc-sfu 端口直推；不引入 jsmpeg 第二链路</t>
+  </si>
+  <si>
+    <t>M-MC-01</t>
+  </si>
+  <si>
+    <t>执行终端接入与台账</t>
+  </si>
+  <si>
+    <t>R-MC-001</t>
+  </si>
+  <si>
+    <t>真机接入与台账（3-8台）</t>
+  </si>
+  <si>
+    <t>演示核心资源池</t>
+  </si>
+  <si>
+    <t>群控管理服务</t>
+  </si>
+  <si>
+    <t>F-MC-01-01</t>
+  </si>
+  <si>
+    <t>移动端终端接入与台账</t>
+  </si>
+  <si>
+    <t>真机 ADB/无障碍接入注册+台账+在线状态</t>
+  </si>
+  <si>
     <t>P1</t>
   </si>
   <si>
-    <t>M-MC-15</t>
-  </si>
-  <si>
-    <t>真机Agent运行时与编排(AI可用)</t>
-  </si>
-  <si>
-    <t>R-MC-015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      </t>
-  </si>
-  <si>
-    <t>CON-15 Agent 独立部署单元；借鉴 SonicCloudOrg(已archived,Apache2.0)；真机=Android 3-8台</t>
-  </si>
-  <si>
-    <t>分布式真机控制服务</t>
-  </si>
-  <si>
-    <t>F-MC-15-01</t>
-  </si>
-  <si>
-    <t>Agent注册与鉴权握手</t>
-  </si>
-  <si>
-    <t>Agent 启动经 II-02 WS 连中心侧编排器，agentKey 配置文件校验 + 版本/能力上报(auth消息)；中心侧回 authResult 分配 agentId</t>
-  </si>
-  <si>
-    <t>杨志</t>
-  </si>
-  <si>
-    <t>agentKey 配置文件读，不做密钥轮换</t>
-  </si>
-  <si>
-    <t>F-MC-15-02</t>
-  </si>
-  <si>
-    <t>心跳保活与在线状态判定</t>
-  </si>
-  <si>
-    <t>Agent 周期发 heartBeat(默认30s)，超时(默认90s)判掉线；推 terminal_offline 事件给 M-MC-01 更新台账在线状态</t>
-  </si>
-  <si>
-    <t>MC-02</t>
-  </si>
-  <si>
-    <t>台账在线状态数据源</t>
-  </si>
-  <si>
-    <t>F-MC-15-03</t>
-  </si>
-  <si>
-    <t>设备占用锁</t>
-  </si>
-  <si>
-    <t>设备占用锁(occupy/release)，一台设备同时只让一个会话用(远控/自动化互斥)；内存锁(单 mc-service 副本)，不做分布式锁</t>
-  </si>
-  <si>
-    <t>防远控和自动化并发打架；分布式锁留 V1.2</t>
-  </si>
-  <si>
-    <t>F-MC-15-04</t>
-  </si>
-  <si>
-    <t>ADB控制通道</t>
-  </si>
-  <si>
-    <t>ddmlib 实现 ADB 通道：install/uninstall/pressKey/reboot/screenshot；动作子集(不做交互式 shell 终端)；经 runAction 消息收口(与 F-MC-15-05 共享)</t>
-  </si>
-  <si>
-    <t>Sonic AndroidDeviceBridgeTool 对应</t>
-  </si>
-  <si>
-    <t>F-MC-15-05</t>
-  </si>
-  <si>
-    <t>无障碍控制通道(uia2)</t>
-  </si>
-  <si>
-    <t>引 sonic-driver-core(Maven jar) 封装 uiautomator2-server：UI 元素 find/click/sendKeys/swipe；断言类步骤全砍；经 runAction 消息收口</t>
-  </si>
-  <si>
-    <t>依赖 archived 库 sonic-driver-core；uia2 协议本身稳定</t>
-  </si>
-  <si>
-    <t>F-MC-15-06</t>
-  </si>
-  <si>
-    <t>远控画面源(scrcpy)</t>
-  </si>
-  <si>
-    <t>抄 Sonic ScrcpyInputSocketThread/OutputSocketThread(Apache2.0)；启动 scrcpy server 抓 H.264 → 经 startScrcpy 推到 mc-sfu 指定端口；本功能只产画面源，WebRTC 转发由 M-MC-04 mc-sfu 承担</t>
-  </si>
-  <si>
-    <t>MC-17</t>
-  </si>
-  <si>
-    <t>媒体面 Agent→mc-sfu 端口直推；不引入 jsmpeg 第二链路</t>
-  </si>
-  <si>
-    <t>M-MC-01</t>
-  </si>
-  <si>
-    <t>执行终端接入与台账</t>
-  </si>
-  <si>
-    <t>R-MC-001</t>
-  </si>
-  <si>
-    <t>真机接入与台账（3-8台）</t>
-  </si>
-  <si>
-    <t>演示核心资源池</t>
-  </si>
-  <si>
-    <t>群控管理服务</t>
-  </si>
-  <si>
-    <t>F-MC-01-01</t>
-  </si>
-  <si>
-    <t>移动端终端接入与台账</t>
-  </si>
-  <si>
-    <t>真机 ADB/无障碍接入注册+台账+在线状态</t>
-  </si>
-  <si>
     <t>全栈</t>
   </si>
   <si>
@@ -320,88 +320,88 @@
     <t>批量截图/状态查询</t>
   </si>
   <si>
+    <t>EI-04</t>
+  </si>
+  <si>
+    <t>F-MC-03-01</t>
+  </si>
+  <si>
+    <t>终端状态与指标监控</t>
+  </si>
+  <si>
+    <t>R-MC-003</t>
+  </si>
+  <si>
+    <t>在线/离线状态</t>
+  </si>
+  <si>
+    <t>MC-01/MC-02</t>
+  </si>
+  <si>
+    <t>F-MC-02-02</t>
+  </si>
+  <si>
+    <t>移动端设备指纹管理</t>
+  </si>
+  <si>
+    <t>R-MC-002</t>
+  </si>
+  <si>
+    <t>真机指纹只读记录</t>
+  </si>
+  <si>
+    <t>真机指纹天然真实</t>
+  </si>
+  <si>
+    <t>F-MC-09-02</t>
+  </si>
+  <si>
+    <t>账号-终端-代理绑定自动化</t>
+  </si>
+  <si>
+    <t>R-MC-009</t>
+  </si>
+  <si>
+    <t>账号-终端-代理绑定自动化（BindingAutomator），写 mc_binding(account_id+terminal_id+proxy_id) 单一存储</t>
+  </si>
+  <si>
+    <t>F-MC-03-04/F-MC-11-01</t>
+  </si>
+  <si>
+    <t>写mc_binding单一存储；CON-13差异化绑定</t>
+  </si>
+  <si>
+    <t>F-MC-09-03</t>
+  </si>
+  <si>
+    <t>终端侧登录状态维护</t>
+  </si>
+  <si>
+    <t>登录态保持</t>
+  </si>
+  <si>
+    <t>M-MC-03</t>
+  </si>
+  <si>
+    <t>终端风控分级与代理绑定</t>
+  </si>
+  <si>
+    <t>终端风控分级+代理绑定（写 mc_binding 网络层侧面 terminal_id+proxy_id）</t>
+  </si>
+  <si>
+    <t>CON-13 绑定规则</t>
+  </si>
+  <si>
+    <t>F-MC-03-04</t>
+  </si>
+  <si>
+    <t>代理分配与固定绑定</t>
+  </si>
+  <si>
+    <t>真机绑定固定代理IP，写 mc_binding(terminal_id+proxy_id) 单一存储</t>
+  </si>
+  <si>
     <t>P2</t>
-  </si>
-  <si>
-    <t>EI-04</t>
-  </si>
-  <si>
-    <t>F-MC-03-01</t>
-  </si>
-  <si>
-    <t>终端状态与指标监控</t>
-  </si>
-  <si>
-    <t>R-MC-003</t>
-  </si>
-  <si>
-    <t>在线/离线状态</t>
-  </si>
-  <si>
-    <t>MC-01/MC-02</t>
-  </si>
-  <si>
-    <t>F-MC-02-02</t>
-  </si>
-  <si>
-    <t>移动端设备指纹管理</t>
-  </si>
-  <si>
-    <t>R-MC-002</t>
-  </si>
-  <si>
-    <t>真机指纹只读记录</t>
-  </si>
-  <si>
-    <t>真机指纹天然真实</t>
-  </si>
-  <si>
-    <t>F-MC-09-02</t>
-  </si>
-  <si>
-    <t>账号-终端-代理绑定自动化</t>
-  </si>
-  <si>
-    <t>R-MC-009</t>
-  </si>
-  <si>
-    <t>账号-终端-代理绑定自动化（BindingAutomator），写 mc_binding(account_id+terminal_id+proxy_id) 单一存储</t>
-  </si>
-  <si>
-    <t>F-MC-03-04/F-MC-11-01</t>
-  </si>
-  <si>
-    <t>写mc_binding单一存储；CON-13差异化绑定</t>
-  </si>
-  <si>
-    <t>F-MC-09-03</t>
-  </si>
-  <si>
-    <t>终端侧登录状态维护</t>
-  </si>
-  <si>
-    <t>登录态保持</t>
-  </si>
-  <si>
-    <t>M-MC-03</t>
-  </si>
-  <si>
-    <t>终端风控分级与代理绑定</t>
-  </si>
-  <si>
-    <t>终端风控分级+代理绑定（写 mc_binding 网络层侧面 terminal_id+proxy_id）</t>
-  </si>
-  <si>
-    <t>CON-13 绑定规则</t>
-  </si>
-  <si>
-    <t>F-MC-03-04</t>
-  </si>
-  <si>
-    <t>代理分配与固定绑定</t>
-  </si>
-  <si>
-    <t>真机绑定固定代理IP，写 mc_binding(terminal_id+proxy_id) 单一存储</t>
   </si>
   <si>
     <t>MC-05(V1.1)</t>
@@ -3865,20 +3865,18 @@
       <c r="G5" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="H5" s="6"/>
+      <c r="I5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M5" s="5" t="s">
         <v>25</v>
@@ -3913,10 +3911,10 @@
         <v>32</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K6">
         <v>3</v>
@@ -3925,7 +3923,7 @@
         <v>33</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N6" s="7" t="s">
         <v>34</v>
@@ -3954,7 +3952,7 @@
         <v>32</v>
       </c>
       <c r="I7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J7" s="7" t="s">
         <v>29</v>
@@ -3966,7 +3964,7 @@
         <v>33</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N7" s="7" t="s">
         <v>25</v>
@@ -3995,7 +3993,7 @@
         <v>32</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J8" s="7" t="s">
         <v>29</v>
@@ -4033,7 +4031,7 @@
         <v>45</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="I9" s="7"/>
       <c r="J9" s="7" t="s">
@@ -4046,7 +4044,7 @@
         <v>33</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N9" s="7" t="s">
         <v>25</v>
@@ -4058,38 +4056,36 @@
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="D10" s="23" t="s">
+      <c r="E10" s="5" t="s">
         <v>48</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>49</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M10" s="5"/>
       <c r="N10" s="5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" ht="36" customHeight="1" spans="1:14">
@@ -4097,28 +4093,28 @@
         <v>27</v>
       </c>
       <c r="B11" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" t="s">
         <v>52</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>53</v>
       </c>
-      <c r="D11" t="s">
-        <v>54</v>
-      </c>
       <c r="E11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F11" t="s">
         <v>21</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="H11" t="s">
+        <v>54</v>
+      </c>
+      <c r="H11" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J11" t="s">
         <v>29</v>
@@ -4127,10 +4123,10 @@
         <v>2</v>
       </c>
       <c r="L11" t="s">
+        <v>55</v>
+      </c>
+      <c r="N11" t="s">
         <v>56</v>
-      </c>
-      <c r="N11" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="12" ht="36" customHeight="1" spans="1:14">
@@ -4138,40 +4134,40 @@
         <v>27</v>
       </c>
       <c r="C12" t="s">
+        <v>57</v>
+      </c>
+      <c r="D12" t="s">
         <v>58</v>
       </c>
-      <c r="D12" t="s">
-        <v>59</v>
-      </c>
       <c r="E12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F12" t="s">
         <v>21</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H12" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K12">
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M12" t="s">
+        <v>60</v>
+      </c>
+      <c r="N12" t="s">
         <v>61</v>
-      </c>
-      <c r="N12" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="13" ht="36" customHeight="1" spans="1:14">
@@ -4179,37 +4175,37 @@
         <v>27</v>
       </c>
       <c r="C13" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" t="s">
         <v>63</v>
       </c>
-      <c r="D13" t="s">
-        <v>64</v>
-      </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F13" t="s">
         <v>21</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>65</v>
-      </c>
-      <c r="H13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H13" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K13">
         <v>2</v>
       </c>
       <c r="L13" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" ht="36" customHeight="1" spans="1:14">
@@ -4217,37 +4213,37 @@
         <v>27</v>
       </c>
       <c r="C14" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" t="s">
         <v>67</v>
       </c>
-      <c r="D14" t="s">
-        <v>68</v>
-      </c>
       <c r="E14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F14" t="s">
         <v>21</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="H14" t="s">
+        <v>68</v>
+      </c>
+      <c r="H14" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K14">
         <v>2</v>
       </c>
       <c r="L14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1" spans="1:14">
@@ -4255,37 +4251,37 @@
         <v>27</v>
       </c>
       <c r="C15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" t="s">
         <v>71</v>
       </c>
-      <c r="D15" t="s">
-        <v>72</v>
-      </c>
       <c r="E15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F15" t="s">
         <v>21</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15" t="s">
+        <v>72</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K15">
         <v>2</v>
       </c>
       <c r="L15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="N15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" ht="48" customHeight="1" spans="1:14">
@@ -4293,40 +4289,40 @@
         <v>27</v>
       </c>
       <c r="C16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" t="s">
         <v>75</v>
       </c>
-      <c r="D16" t="s">
-        <v>76</v>
-      </c>
       <c r="E16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F16" t="s">
         <v>21</v>
       </c>
       <c r="G16" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="H16" t="s">
+        <v>76</v>
+      </c>
+      <c r="H16" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J16" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K16">
         <v>2</v>
       </c>
       <c r="L16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M16" t="s">
+        <v>77</v>
+      </c>
+      <c r="N16" t="s">
         <v>78</v>
-      </c>
-      <c r="N16" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="17" ht="40" customHeight="1" spans="1:14">
@@ -4335,40 +4331,38 @@
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>81</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>82</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="H17" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="6"/>
+      <c r="I17" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>29</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M17" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N17" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" ht="40" customHeight="1" spans="1:14">
@@ -4376,25 +4370,25 @@
         <v>27</v>
       </c>
       <c r="B18" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="C18" s="7" t="s">
+      <c r="D18" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>87</v>
-      </c>
       <c r="E18" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F18" s="7" t="s">
         <v>21</v>
       </c>
       <c r="G18" s="8" t="s">
+        <v>87</v>
+      </c>
+      <c r="H18" s="8" t="s">
         <v>88</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>32</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>89</v>
@@ -4409,7 +4403,7 @@
         <v>90</v>
       </c>
       <c r="M18" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N18" s="7" t="s">
         <v>91</v>
@@ -4426,7 +4420,7 @@
         <v>93</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F19" s="7" t="s">
         <v>21</v>
@@ -4435,13 +4429,13 @@
         <v>94</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>89</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K19">
         <v>1</v>
@@ -4450,10 +4444,10 @@
         <v>90</v>
       </c>
       <c r="M19" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N19" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="20" ht="40" customHeight="1" spans="1:14">
@@ -4461,28 +4455,28 @@
         <v>27</v>
       </c>
       <c r="C20" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="D20" s="12" t="s">
+      <c r="E20" s="12" t="s">
         <v>98</v>
-      </c>
-      <c r="E20" s="12" t="s">
-        <v>99</v>
       </c>
       <c r="F20" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="H20" s="13" t="s">
-        <v>46</v>
+        <v>99</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="I20" s="11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K20">
         <v>1</v>
@@ -4491,7 +4485,7 @@
         <v>90</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="N20" s="7" t="s">
         <v>25</v>
@@ -4502,28 +4496,28 @@
         <v>27</v>
       </c>
       <c r="C21" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="12" t="s">
         <v>103</v>
-      </c>
-      <c r="E21" s="12" t="s">
-        <v>104</v>
       </c>
       <c r="F21" s="12" t="s">
         <v>21</v>
       </c>
       <c r="G21" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="H21" s="13" t="s">
-        <v>95</v>
+        <v>104</v>
+      </c>
+      <c r="H21" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="I21" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K21">
         <v>1</v>
@@ -4532,10 +4526,10 @@
         <v>90</v>
       </c>
       <c r="M21" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N21" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" ht="40" customHeight="1" spans="1:14">
@@ -4543,28 +4537,28 @@
         <v>27</v>
       </c>
       <c r="C22" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="E22" s="7" t="s">
         <v>108</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>109</v>
       </c>
       <c r="F22" s="7" t="s">
         <v>21</v>
       </c>
       <c r="G22" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="H22" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J22" s="7" t="s">
         <v>110</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>111</v>
       </c>
       <c r="K22">
         <v>1</v>
@@ -4573,10 +4567,10 @@
         <v>90</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N22" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" ht="40" customHeight="1" spans="1:14">
@@ -4584,28 +4578,28 @@
         <v>27</v>
       </c>
       <c r="C23" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="D23" s="7" t="s">
-        <v>114</v>
-      </c>
       <c r="E23" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>21</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K23">
         <v>1</v>
@@ -4614,7 +4608,7 @@
         <v>90</v>
       </c>
       <c r="M23" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N23" s="7" t="s">
         <v>25</v>
@@ -4626,40 +4620,38 @@
       </c>
       <c r="B24" s="22"/>
       <c r="C24" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D24" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="5" t="s">
-        <v>117</v>
-      </c>
       <c r="E24" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F24" s="5" t="s">
         <v>21</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="H24" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="H24" s="6"/>
+      <c r="I24" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I24" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="J24" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>25</v>
       </c>
       <c r="N24" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" ht="40" customHeight="1" spans="1:14">
@@ -4667,31 +4659,31 @@
         <v>27</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C25" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>121</v>
-      </c>
       <c r="E25" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F25" s="7" t="s">
         <v>21</v>
       </c>
       <c r="G25" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="H25" s="8" t="s">
         <v>122</v>
       </c>
-      <c r="H25" s="8" t="s">
-        <v>46</v>
-      </c>
       <c r="I25" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K25">
         <v>1</v>
@@ -4717,7 +4709,7 @@
         <v>126</v>
       </c>
       <c r="E26" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F26" s="7" t="s">
         <v>127</v>
@@ -4726,13 +4718,13 @@
         <v>128</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>46</v>
+        <v>122</v>
       </c>
       <c r="I26" s="26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K26">
         <v>1</v>
@@ -4767,20 +4759,18 @@
       <c r="G27" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="H27" s="6" t="s">
+      <c r="H27" s="6"/>
+      <c r="I27" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I27" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J27" s="5" t="s">
         <v>135</v>
       </c>
       <c r="K27" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M27" s="5" t="s">
         <v>25</v>
@@ -4794,7 +4784,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C28" s="7" t="s">
         <v>137</v>
@@ -4818,16 +4808,16 @@
         <v>89</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K28">
         <v>2</v>
       </c>
       <c r="L28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M28" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N28" s="7" t="s">
         <v>140</v>
@@ -4865,7 +4855,7 @@
         <v>2</v>
       </c>
       <c r="L29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="M29" s="7" t="s">
         <v>144</v>
@@ -4894,20 +4884,18 @@
       <c r="G30" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="6"/>
+      <c r="I30" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I30" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J30" s="5" t="s">
         <v>29</v>
       </c>
       <c r="K30" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M30" s="5" t="s">
         <v>25</v>
@@ -4921,7 +4909,7 @@
         <v>27</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C31" s="7" t="s">
         <v>151</v>
@@ -4942,7 +4930,7 @@
         <v>32</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>29</v>
@@ -4983,7 +4971,7 @@
         <v>32</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>29</v>
@@ -5021,20 +5009,18 @@
       <c r="G33" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="H33" s="6" t="s">
+      <c r="H33" s="6"/>
+      <c r="I33" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="I33" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="J33" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K33" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M33" s="5" t="s">
         <v>25</v>
@@ -5048,7 +5034,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C34" s="7" t="s">
         <v>166</v>
@@ -5066,13 +5052,13 @@
         <v>168</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>46</v>
+        <v>122</v>
       </c>
       <c r="I34" s="7" t="s">
         <v>89</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K34">
         <v>2</v>
@@ -5107,7 +5093,7 @@
         <v>173</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>89</v>
@@ -5147,11 +5133,11 @@
       <c r="G36" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="H36" s="13" t="s">
-        <v>95</v>
+      <c r="H36" s="8" t="s">
+        <v>122</v>
       </c>
       <c r="I36" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J36" s="12" t="s">
         <v>171</v>
@@ -5163,7 +5149,7 @@
         <v>90</v>
       </c>
       <c r="M36" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N36" s="7" t="s">
         <v>178</v>
@@ -5189,20 +5175,18 @@
       <c r="G37" s="27" t="s">
         <v>182</v>
       </c>
-      <c r="H37" s="6" t="s">
+      <c r="H37" s="6"/>
+      <c r="I37" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I37" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J37" s="5" t="s">
         <v>166</v>
       </c>
       <c r="K37" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M37" s="5" t="s">
         <v>25</v>
@@ -5234,13 +5218,13 @@
         <v>187</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>46</v>
+        <v>122</v>
       </c>
       <c r="I38" s="7" t="s">
         <v>89</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K38">
         <v>2</v>
@@ -5275,7 +5259,7 @@
         <v>192</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I39" s="7" t="s">
         <v>89</v>
@@ -5316,20 +5300,18 @@
       <c r="G40" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="H40" s="6" t="s">
+      <c r="H40" s="6"/>
+      <c r="I40" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I40" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J40" s="5" t="s">
         <v>29</v>
       </c>
       <c r="K40" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M40" s="5" t="s">
         <v>25</v>
@@ -5343,7 +5325,7 @@
         <v>27</v>
       </c>
       <c r="B41" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C41" s="7" t="s">
         <v>199</v>
@@ -5361,7 +5343,7 @@
         <v>201</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="I41" s="7" t="s">
         <v>89</v>
@@ -5402,7 +5384,7 @@
         <v>205</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I42" s="7" t="s">
         <v>89</v>
@@ -5442,8 +5424,8 @@
       <c r="G43" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="H43" s="13" t="s">
-        <v>32</v>
+      <c r="H43" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="I43" s="12" t="s">
         <v>89</v>
@@ -5484,7 +5466,7 @@
         <v>212</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I44" s="7" t="s">
         <v>89</v>
@@ -5525,20 +5507,18 @@
       <c r="G45" s="6" t="s">
         <v>216</v>
       </c>
-      <c r="H45" s="6" t="s">
+      <c r="H45" s="6"/>
+      <c r="I45" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I45" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J45" s="5" t="s">
         <v>38</v>
       </c>
       <c r="K45" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M45" s="5" t="s">
         <v>25</v>
@@ -5552,7 +5532,7 @@
         <v>27</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C46" s="7" t="s">
         <v>218</v>
@@ -5570,10 +5550,10 @@
         <v>220</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="I46" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J46" s="7" t="s">
         <v>38</v>
@@ -5611,10 +5591,10 @@
         <v>223</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I47" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J47" s="7" t="s">
         <v>218</v>
@@ -5652,10 +5632,10 @@
         <v>226</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I48" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J48" s="7" t="s">
         <v>218</v>
@@ -5692,11 +5672,11 @@
       <c r="G49" s="13" t="s">
         <v>229</v>
       </c>
-      <c r="H49" s="13" t="s">
-        <v>32</v>
+      <c r="H49" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="I49" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J49" s="12" t="s">
         <v>218</v>
@@ -5708,7 +5688,7 @@
         <v>90</v>
       </c>
       <c r="M49" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N49" s="7" t="s">
         <v>230</v>
@@ -5734,7 +5714,7 @@
         <v>233</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="I50" s="7" t="s">
         <v>89</v>
@@ -5776,19 +5756,19 @@
         <v>238</v>
       </c>
       <c r="H51" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I51" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I51" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J51" s="5" t="s">
         <v>239</v>
       </c>
       <c r="K51" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L51" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M51" s="5" t="s">
         <v>25</v>
@@ -5861,7 +5841,7 @@
         <v>247</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I53" s="7" t="s">
         <v>89</v>
@@ -5905,7 +5885,7 @@
         <v>32</v>
       </c>
       <c r="I54" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J54" s="7" t="s">
         <v>252</v>
@@ -5984,7 +5964,7 @@
         <v>259</v>
       </c>
       <c r="H56" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I56" s="7" t="s">
         <v>260</v>
@@ -6026,19 +6006,19 @@
         <v>265</v>
       </c>
       <c r="H57" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I57" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I57" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J57" s="5" t="s">
         <v>199</v>
       </c>
       <c r="K57" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L57" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M57" s="5" t="s">
         <v>25</v>
@@ -6052,7 +6032,7 @@
         <v>27</v>
       </c>
       <c r="B58" s="24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C58" s="7" t="s">
         <v>267</v>
@@ -6070,7 +6050,7 @@
         <v>269</v>
       </c>
       <c r="H58" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I58" s="7" t="s">
         <v>89</v>
@@ -6109,7 +6089,7 @@
         <v>275</v>
       </c>
       <c r="H59" s="13" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I59" s="12" t="s">
         <v>89</v>
@@ -6145,7 +6125,7 @@
         <v>280</v>
       </c>
       <c r="H60" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="I60" s="7" t="s">
         <v>89</v>
@@ -6172,7 +6152,7 @@
         <v>283</v>
       </c>
       <c r="E61" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F61" s="7" t="s">
         <v>127</v>
@@ -6181,13 +6161,13 @@
         <v>284</v>
       </c>
       <c r="H61" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I61" s="7" t="s">
         <v>89</v>
       </c>
       <c r="J61" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L61" s="11"/>
       <c r="M61" s="7" t="s">
@@ -6217,7 +6197,7 @@
         <v>288</v>
       </c>
       <c r="H62" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I62" s="7" t="s">
         <v>89</v>
@@ -6253,7 +6233,7 @@
         <v>291</v>
       </c>
       <c r="H63" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I63" s="7" t="s">
         <v>89</v>
@@ -6285,7 +6265,7 @@
         <v>294</v>
       </c>
       <c r="E65" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F65" s="7" t="s">
         <v>295</v>
@@ -6294,18 +6274,18 @@
         <v>296</v>
       </c>
       <c r="H65" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I65" s="7" t="s">
         <v>89</v>
       </c>
       <c r="J65" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="K65" s="7"/>
       <c r="L65" s="7"/>
       <c r="M65" s="7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="N65" s="7" t="s">
         <v>297</v>
@@ -6322,7 +6302,7 @@
         <v>299</v>
       </c>
       <c r="E66" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F66" s="7" t="s">
         <v>295</v>
@@ -6331,10 +6311,10 @@
         <v>300</v>
       </c>
       <c r="H66" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I66" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J66" s="7" t="s">
         <v>293</v>
@@ -6342,7 +6322,7 @@
       <c r="K66" s="7"/>
       <c r="L66" s="7"/>
       <c r="M66" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N66" s="7" t="s">
         <v>301</v>
@@ -6359,7 +6339,7 @@
         <v>303</v>
       </c>
       <c r="E67" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F67" s="7" t="s">
         <v>295</v>
@@ -6368,10 +6348,10 @@
         <v>304</v>
       </c>
       <c r="H67" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I67" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J67" s="7" t="s">
         <v>305</v>
@@ -6379,7 +6359,7 @@
       <c r="K67" s="7"/>
       <c r="L67" s="7"/>
       <c r="M67" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N67" s="7" t="s">
         <v>304</v>
@@ -6405,7 +6385,7 @@
         <v>308</v>
       </c>
       <c r="H68" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I68" s="7" t="s">
         <v>89</v>
@@ -6416,7 +6396,7 @@
       <c r="K68" s="7"/>
       <c r="L68" s="7"/>
       <c r="M68" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N68" s="7" t="s">
         <v>301</v>
@@ -6442,7 +6422,7 @@
         <v>310</v>
       </c>
       <c r="H69" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I69" s="7" t="s">
         <v>89</v>
@@ -6453,7 +6433,7 @@
       <c r="K69" s="7"/>
       <c r="L69" s="7"/>
       <c r="M69" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N69" s="7" t="s">
         <v>25</v>
@@ -6470,7 +6450,7 @@
         <v>312</v>
       </c>
       <c r="E70" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="F70" s="7" t="s">
         <v>295</v>
@@ -6479,18 +6459,18 @@
         <v>313</v>
       </c>
       <c r="H70" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I70" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J70" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K70" s="7"/>
       <c r="L70" s="7"/>
       <c r="M70" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N70" s="7" t="s">
         <v>25</v>
@@ -6516,7 +6496,7 @@
         <v>316</v>
       </c>
       <c r="H71" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I71" s="7" t="s">
         <v>89</v>
@@ -6553,7 +6533,7 @@
         <v>319</v>
       </c>
       <c r="H72" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I72" s="7" t="s">
         <v>89</v>
@@ -6591,7 +6571,7 @@
         <v>322</v>
       </c>
       <c r="H73" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I73" s="12" t="s">
         <v>89</v>
@@ -6628,7 +6608,7 @@
         <v>325</v>
       </c>
       <c r="H74" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I74" s="7" t="s">
         <v>89</v>
@@ -6666,17 +6646,17 @@
         <v>329</v>
       </c>
       <c r="H75" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="I75" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="I75" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="J75" s="5" t="s">
         <v>185</v>
       </c>
       <c r="K75" s="5"/>
       <c r="L75" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M75" s="5" t="s">
         <v>25</v>
@@ -6705,7 +6685,7 @@
         <v>331</v>
       </c>
       <c r="H76" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I76" s="7" t="s">
         <v>89</v>
@@ -6742,7 +6722,7 @@
         <v>334</v>
       </c>
       <c r="H77" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I77" s="7" t="s">
         <v>89</v>
@@ -6779,10 +6759,10 @@
         <v>337</v>
       </c>
       <c r="H78" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I78" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J78" s="7" t="s">
         <v>190</v>
@@ -6790,7 +6770,7 @@
       <c r="K78" s="7"/>
       <c r="L78" s="7"/>
       <c r="M78" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N78" s="7" t="s">
         <v>25</v>
@@ -6816,10 +6796,10 @@
         <v>340</v>
       </c>
       <c r="H79" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I79" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J79" s="7" t="s">
         <v>335</v>
@@ -6827,7 +6807,7 @@
       <c r="K79" s="7"/>
       <c r="L79" s="7"/>
       <c r="M79" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N79" s="7" t="s">
         <v>25</v>
@@ -6853,10 +6833,10 @@
         <v>343</v>
       </c>
       <c r="H80" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I80" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J80" s="7" t="s">
         <v>338</v>
@@ -6864,7 +6844,7 @@
       <c r="K80" s="7"/>
       <c r="L80" s="7"/>
       <c r="M80" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N80" s="7" t="s">
         <v>25</v>
@@ -6890,7 +6870,7 @@
         <v>346</v>
       </c>
       <c r="H81" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I81" s="7" t="s">
         <v>89</v>
@@ -6932,22 +6912,22 @@
         <v>351</v>
       </c>
       <c r="H83" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="I83" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J83" s="7" t="s">
         <v>278</v>
       </c>
       <c r="K83" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L83" s="7" t="s">
         <v>352</v>
       </c>
       <c r="M83" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N83" s="7" t="s">
         <v>353</v>
@@ -7079,19 +7059,19 @@
         <v>360</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="I5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>25</v>
@@ -7120,13 +7100,13 @@
         <v>364</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J6">
         <v>8</v>
@@ -7135,7 +7115,7 @@
         <v>365</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>366</v>
@@ -7161,10 +7141,10 @@
         <v>370</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>362</v>
@@ -7176,7 +7156,7 @@
         <v>365</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>25</v>
@@ -7202,19 +7182,19 @@
         <v>374</v>
       </c>
       <c r="G8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I8" s="5" t="s">
         <v>362</v>
       </c>
       <c r="J8" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K8" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L8" s="5" t="s">
         <v>25</v>
@@ -7243,22 +7223,22 @@
         <v>378</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>362</v>
       </c>
       <c r="J9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K9" s="7" t="s">
         <v>365</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>379</v>
@@ -7284,22 +7264,22 @@
         <v>383</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>375</v>
       </c>
       <c r="J10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>365</v>
       </c>
       <c r="L10" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>384</v>
@@ -7330,22 +7310,22 @@
         <v>388</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>362</v>
       </c>
       <c r="J12">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>365</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>25</v>
@@ -7371,10 +7351,10 @@
         <v>391</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>385</v>
@@ -7386,7 +7366,7 @@
         <v>365</v>
       </c>
       <c r="L13" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>25</v>
@@ -7412,10 +7392,10 @@
         <v>394</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>385</v>
@@ -7427,7 +7407,7 @@
         <v>365</v>
       </c>
       <c r="L14" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>25</v>
@@ -7453,10 +7433,10 @@
         <v>396</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>392</v>
@@ -7468,7 +7448,7 @@
         <v>365</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>25</v>
@@ -7494,22 +7474,22 @@
         <v>399</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>400</v>
       </c>
       <c r="J16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" s="17" t="s">
         <v>401</v>
       </c>
       <c r="L16" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>25</v>
@@ -7535,22 +7515,22 @@
         <v>402</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K17" s="17" t="s">
         <v>401</v>
       </c>
       <c r="L17" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M17" s="7" t="s">
         <v>25</v>
@@ -7576,22 +7556,22 @@
         <v>405</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>367</v>
       </c>
       <c r="J18">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>365</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>25</v>
@@ -7653,19 +7633,19 @@
         <v>413</v>
       </c>
       <c r="G21" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H21" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H21" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I21" s="5" t="s">
         <v>414</v>
       </c>
       <c r="J21" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L21" s="5" t="s">
         <v>25</v>
@@ -7694,10 +7674,10 @@
         <v>418</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H22" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>419</v>
@@ -7709,7 +7689,7 @@
         <v>420</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>25</v>
@@ -7826,19 +7806,19 @@
         <v>426</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="I5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>25</v>
@@ -7867,13 +7847,13 @@
         <v>430</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -7882,7 +7862,7 @@
         <v>365</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>431</v>
@@ -7908,16 +7888,16 @@
         <v>435</v>
       </c>
       <c r="G7" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>428</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L7" s="5" t="s">
         <v>25</v>
@@ -7946,7 +7926,7 @@
         <v>439</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>89</v>
@@ -7961,7 +7941,7 @@
         <v>365</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M8" s="7" t="s">
         <v>440</v>
@@ -7992,10 +7972,10 @@
         <v>444</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>428</v>
@@ -8003,7 +7983,7 @@
       <c r="J10" s="7"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>445</v>
@@ -8029,19 +8009,19 @@
         <v>448</v>
       </c>
       <c r="G11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="I11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L11" s="5" t="s">
         <v>25</v>
@@ -8070,18 +8050,18 @@
         <v>452</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J12" s="7"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>453</v>
@@ -8107,10 +8087,10 @@
         <v>456</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>450</v>
@@ -8118,7 +8098,7 @@
       <c r="J13" s="7"/>
       <c r="K13" s="7"/>
       <c r="L13" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M13" s="7" t="s">
         <v>25</v>
@@ -8144,19 +8124,19 @@
         <v>459</v>
       </c>
       <c r="G14" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I14" s="5" t="s">
         <v>450</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L14" s="5" t="s">
         <v>25</v>
@@ -8185,10 +8165,10 @@
         <v>463</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>450</v>
@@ -8196,7 +8176,7 @@
       <c r="J15" s="7"/>
       <c r="K15" s="11"/>
       <c r="L15" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>464</v>
@@ -8222,10 +8202,10 @@
         <v>467</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>461</v>
@@ -8235,7 +8215,7 @@
       </c>
       <c r="K16" s="7"/>
       <c r="L16" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>25</v>
@@ -8266,10 +8246,10 @@
         <v>471</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>437</v>
@@ -8277,7 +8257,7 @@
       <c r="J18" s="7"/>
       <c r="K18" s="7"/>
       <c r="L18" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>25</v>
@@ -8397,19 +8377,19 @@
         <v>478</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="I5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>25</v>
@@ -8438,13 +8418,13 @@
         <v>482</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J6">
         <v>5</v>
@@ -8479,10 +8459,10 @@
         <v>487</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>480</v>
@@ -8494,7 +8474,7 @@
         <v>483</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>488</v>
@@ -8520,7 +8500,7 @@
         <v>491</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>89</v>
@@ -8561,7 +8541,7 @@
         <v>496</v>
       </c>
       <c r="G9" s="13" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H9" s="12" t="s">
         <v>260</v>
@@ -8602,16 +8582,16 @@
         <v>500</v>
       </c>
       <c r="G10" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I10" s="5" t="s">
         <v>480</v>
       </c>
       <c r="K10" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L10" s="5" t="s">
         <v>25</v>
@@ -8640,10 +8620,10 @@
         <v>503</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>480</v>
@@ -8655,7 +8635,7 @@
         <v>483</v>
       </c>
       <c r="L11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>504</v>
@@ -8681,10 +8661,10 @@
         <v>507</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>501</v>
@@ -8696,7 +8676,7 @@
         <v>483</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>508</v>
@@ -8722,7 +8702,7 @@
         <v>511</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>89</v>
@@ -8731,7 +8711,7 @@
         <v>501</v>
       </c>
       <c r="J13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K13" s="7" t="s">
         <v>483</v>
@@ -8763,7 +8743,7 @@
         <v>516</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>89</v>
@@ -8772,7 +8752,7 @@
         <v>501</v>
       </c>
       <c r="J14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>483</v>
@@ -8804,7 +8784,7 @@
         <v>520</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>89</v>
@@ -8813,7 +8793,7 @@
         <v>505</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>483</v>
@@ -8845,7 +8825,7 @@
         <v>524</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>89</v>
@@ -8854,7 +8834,7 @@
         <v>480</v>
       </c>
       <c r="J16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K16" s="7" t="s">
         <v>483</v>
@@ -8886,7 +8866,7 @@
         <v>528</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>89</v>
@@ -8895,7 +8875,7 @@
         <v>480</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>483</v>
@@ -8927,7 +8907,7 @@
         <v>532</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>89</v>
@@ -8936,7 +8916,7 @@
         <v>501</v>
       </c>
       <c r="J18">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>483</v>
@@ -8968,7 +8948,7 @@
         <v>536</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>89</v>
@@ -8977,7 +8957,7 @@
         <v>501</v>
       </c>
       <c r="J19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>483</v>
@@ -9009,16 +8989,16 @@
         <v>540</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>483</v>
@@ -9050,16 +9030,16 @@
         <v>544</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J21">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K21" s="7" t="s">
         <v>483</v>
@@ -9091,16 +9071,16 @@
         <v>548</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K22" s="7" t="s">
         <v>483</v>
@@ -9132,7 +9112,7 @@
         <v>552</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H23" s="7" t="s">
         <v>89</v>
@@ -9141,7 +9121,7 @@
         <v>480</v>
       </c>
       <c r="J23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K23" s="7" t="s">
         <v>483</v>
@@ -9173,7 +9153,7 @@
         <v>556</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>89</v>
@@ -9182,7 +9162,7 @@
         <v>505</v>
       </c>
       <c r="J24">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K24" s="7" t="s">
         <v>483</v>
@@ -9214,22 +9194,22 @@
         <v>559</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>480</v>
       </c>
       <c r="J25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K25" s="7" t="s">
         <v>483</v>
       </c>
       <c r="L25" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>560</v>
@@ -9255,22 +9235,22 @@
         <v>563</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H26" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>501</v>
       </c>
       <c r="J26">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K26" s="7" t="s">
         <v>483</v>
       </c>
       <c r="L26" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>564</v>
@@ -9388,19 +9368,19 @@
         <v>570</v>
       </c>
       <c r="G5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>571</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>25</v>
@@ -9429,13 +9409,13 @@
         <v>575</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J6">
         <v>2</v>
@@ -9511,7 +9491,7 @@
         <v>583</v>
       </c>
       <c r="G8" s="13" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H8" s="12" t="s">
         <v>89</v>
@@ -9552,16 +9532,16 @@
         <v>587</v>
       </c>
       <c r="G9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I9" s="5" t="s">
         <v>571</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L9" s="5" t="s">
         <v>25</v>
@@ -9590,13 +9570,13 @@
         <v>591</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J10">
         <v>2</v>
@@ -9631,7 +9611,7 @@
         <v>596</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>89</v>
@@ -9672,7 +9652,7 @@
         <v>599</v>
       </c>
       <c r="G12" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H12" s="12" t="s">
         <v>89</v>
@@ -9713,16 +9693,16 @@
         <v>605</v>
       </c>
       <c r="G13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="5" t="s">
-        <v>24</v>
-      </c>
       <c r="I13" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L13" s="5" t="s">
         <v>25</v>
@@ -9751,13 +9731,13 @@
         <v>609</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>89</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14">
         <v>3</v>
@@ -9792,10 +9772,10 @@
         <v>613</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H15" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I15" s="12" t="s">
         <v>607</v>
@@ -9807,7 +9787,7 @@
         <v>188</v>
       </c>
       <c r="L15" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M15" s="7" t="s">
         <v>614</v>
@@ -9833,16 +9813,16 @@
         <v>618</v>
       </c>
       <c r="G16" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I16" s="5" t="s">
         <v>577</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L16" s="5" t="s">
         <v>25</v>
@@ -9915,7 +9895,7 @@
         <v>32</v>
       </c>
       <c r="H18" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>620</v>
@@ -9927,7 +9907,7 @@
         <v>188</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>244</v>
@@ -9953,10 +9933,10 @@
         <v>596</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>620</v>
@@ -9968,7 +9948,7 @@
         <v>188</v>
       </c>
       <c r="L19" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>248</v>
@@ -9994,10 +9974,10 @@
         <v>247</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H20" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>620</v>
@@ -10009,7 +9989,7 @@
         <v>188</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>248</v>
@@ -10035,7 +10015,7 @@
         <v>634</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>260</v>
@@ -10081,19 +10061,19 @@
         <v>640</v>
       </c>
       <c r="G23" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="H23" s="5" t="s">
-        <v>24</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>620</v>
       </c>
       <c r="J23" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K23" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L23" s="5" t="s">
         <v>25</v>
@@ -10122,7 +10102,7 @@
         <v>644</v>
       </c>
       <c r="G24" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H24" s="12" t="s">
         <v>89</v>
@@ -10159,7 +10139,7 @@
         <v>649</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>89</v>
@@ -10196,7 +10176,7 @@
         <v>653</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>89</v>
@@ -10233,10 +10213,10 @@
         <v>657</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>651</v>
@@ -10244,7 +10224,7 @@
       <c r="J27" s="7"/>
       <c r="K27" s="7"/>
       <c r="L27" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M27" s="7" t="s">
         <v>25</v>
@@ -10270,10 +10250,10 @@
         <v>660</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H28" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>655</v>
@@ -10281,7 +10261,7 @@
       <c r="J28" s="7"/>
       <c r="K28" s="7"/>
       <c r="L28" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M28" s="7" t="s">
         <v>25</v>
@@ -10307,7 +10287,7 @@
         <v>663</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>260</v>
@@ -10349,10 +10329,10 @@
         <v>667</v>
       </c>
       <c r="G31" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H31" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I31" s="12" t="s">
         <v>607</v>
@@ -10386,10 +10366,10 @@
         <v>670</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>665</v>
@@ -10397,7 +10377,7 @@
       <c r="J32" s="7"/>
       <c r="K32" s="7"/>
       <c r="L32" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M32" s="7" t="s">
         <v>25</v>
@@ -10423,10 +10403,10 @@
         <v>673</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>658</v>
@@ -10434,7 +10414,7 @@
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
       <c r="L33" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M33" s="7" t="s">
         <v>25</v>
@@ -10465,10 +10445,10 @@
         <v>677</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>671</v>
@@ -10476,7 +10456,7 @@
       <c r="J35" s="7"/>
       <c r="K35" s="7"/>
       <c r="L35" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="M35" s="7" t="s">
         <v>678</v>
@@ -10591,16 +10571,16 @@
         <v>684</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>25</v>
@@ -10629,10 +10609,10 @@
         <v>688</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I6">
         <v>3</v>
@@ -10667,7 +10647,7 @@
         <v>694</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>686</v>
@@ -10705,7 +10685,7 @@
         <v>697</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>686</v>
@@ -10743,16 +10723,16 @@
         <v>701</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>702</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>25</v>
@@ -10857,7 +10837,7 @@
         <v>697</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>709</v>
@@ -10895,7 +10875,7 @@
         <v>719</v>
       </c>
       <c r="G13" s="13" t="s">
-        <v>46</v>
+        <v>88</v>
       </c>
       <c r="H13" s="12" t="s">
         <v>686</v>
@@ -10933,16 +10913,16 @@
         <v>725</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H14" s="5" t="s">
         <v>709</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J14" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K14" s="5" t="s">
         <v>25</v>
@@ -10971,7 +10951,7 @@
         <v>728</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>709</v>
@@ -11009,7 +10989,7 @@
         <v>732</v>
       </c>
       <c r="G16" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H16" s="12" t="s">
         <v>726</v>
@@ -11021,7 +11001,7 @@
         <v>689</v>
       </c>
       <c r="K16" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L16" s="7" t="s">
         <v>733</v>
@@ -11047,16 +11027,16 @@
         <v>737</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H17" s="5" t="s">
         <v>726</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J17" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K17" s="5" t="s">
         <v>25</v>
@@ -11083,7 +11063,7 @@
       </c>
       <c r="F18" s="7"/>
       <c r="G18" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>726</v>
@@ -11095,7 +11075,7 @@
         <v>420</v>
       </c>
       <c r="K18" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L18" s="7" t="s">
         <v>742</v>
@@ -11119,7 +11099,7 @@
       </c>
       <c r="F19" s="7"/>
       <c r="G19" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>746</v>
@@ -11131,7 +11111,7 @@
         <v>420</v>
       </c>
       <c r="K19" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L19" s="7" t="s">
         <v>25</v>
@@ -11157,7 +11137,7 @@
         <v>750</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H20" s="12" t="s">
         <v>746</v>
@@ -11169,7 +11149,7 @@
         <v>420</v>
       </c>
       <c r="K20" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L20" s="7" t="s">
         <v>25</v>
@@ -11195,7 +11175,7 @@
         <v>752</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>754</v>
@@ -11207,7 +11187,7 @@
         <v>420</v>
       </c>
       <c r="K21" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L21" s="7" t="s">
         <v>25</v>
@@ -11233,7 +11213,7 @@
         <v>757</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H22" s="12" t="s">
         <v>692</v>
@@ -11276,16 +11256,16 @@
         <v>762</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>25</v>
@@ -11314,15 +11294,15 @@
         <v>766</v>
       </c>
       <c r="G25" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I25" s="7"/>
       <c r="J25" s="11"/>
       <c r="K25" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L25" s="7" t="s">
         <v>25</v>
@@ -11348,14 +11328,14 @@
         <v>770</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I26" s="5"/>
       <c r="J26" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K26" s="5" t="s">
         <v>25</v>
@@ -11384,15 +11364,15 @@
         <v>774</v>
       </c>
       <c r="G27" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="11"/>
       <c r="K27" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L27" s="7" t="s">
         <v>25</v>
@@ -11418,14 +11398,14 @@
         <v>777</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>755</v>
       </c>
       <c r="I28" s="5"/>
       <c r="J28" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K28" s="5" t="s">
         <v>25</v>
@@ -11454,7 +11434,7 @@
         <v>780</v>
       </c>
       <c r="G29" s="13" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H29" s="12" t="s">
         <v>755</v>
@@ -11462,7 +11442,7 @@
       <c r="I29" s="7"/>
       <c r="J29" s="11"/>
       <c r="K29" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L29" s="7" t="s">
         <v>781</v>
@@ -11488,14 +11468,14 @@
         <v>784</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H30" s="5" t="s">
         <v>704</v>
       </c>
       <c r="I30" s="5"/>
       <c r="J30" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K30" s="5" t="s">
         <v>25</v>
@@ -11524,7 +11504,7 @@
         <v>788</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>714</v>
@@ -11532,7 +11512,7 @@
       <c r="I31" s="7"/>
       <c r="J31" s="11"/>
       <c r="K31" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L31" s="7" t="s">
         <v>789</v>
@@ -11647,16 +11627,16 @@
         <v>797</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>25</v>
@@ -11688,14 +11668,14 @@
         <v>32</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I6" s="7">
         <v>7</v>
       </c>
       <c r="J6" s="7"/>
       <c r="K6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L6" s="7" t="s">
         <v>802</v>
@@ -11731,7 +11711,7 @@
       </c>
       <c r="J7" s="7"/>
       <c r="K7" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L7" s="7" t="s">
         <v>806</v>
@@ -11767,7 +11747,7 @@
       </c>
       <c r="J8" s="7"/>
       <c r="K8" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L8" s="7" t="s">
         <v>810</v>
@@ -11798,7 +11778,7 @@
         <v>814</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>803</v>
@@ -11806,7 +11786,7 @@
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
       <c r="K10" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L10" s="7" t="s">
         <v>815</v>
@@ -11832,7 +11812,7 @@
         <v>818</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>803</v>
@@ -11840,7 +11820,7 @@
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
       <c r="K11" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L11" s="7" t="s">
         <v>815</v>
@@ -11866,7 +11846,7 @@
         <v>821</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>803</v>
@@ -11874,7 +11854,7 @@
       <c r="I12" s="7"/>
       <c r="J12" s="7"/>
       <c r="K12" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L12" s="7" t="s">
         <v>815</v>
@@ -11900,7 +11880,7 @@
         <v>823</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>812</v>
@@ -11908,7 +11888,7 @@
       <c r="I13" s="7"/>
       <c r="J13" s="7"/>
       <c r="K13" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>815</v>

</xml_diff>

<commit_message>
vault backup: 2026-07-24 10:01:37
</commit_message>
<xml_diff>
--- a/公司项目/认知行动/文档/MVP功能清单.xlsx
+++ b/公司项目/认知行动/文档/MVP功能清单.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12420" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12420"/>
   </bookViews>
   <sheets>
     <sheet name="MC 多设备矩阵自动化群控子系统" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2322" uniqueCount="824">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2328" uniqueCount="824">
   <si>
     <t>MC 多设备矩阵自动化群控子系统 · 功能清单（V1.0~V1.3）</t>
   </si>
@@ -4872,7 +4872,7 @@
       <c r="C30" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="23" t="s">
         <v>147</v>
       </c>
       <c r="E30" s="5" t="s">
@@ -5288,7 +5288,7 @@
       <c r="C40" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="23" t="s">
         <v>195</v>
       </c>
       <c r="E40" s="5" t="s">
@@ -7856,7 +7856,7 @@
         <v>24</v>
       </c>
       <c r="J6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>365</v>
@@ -7935,7 +7935,7 @@
         <v>428</v>
       </c>
       <c r="J8">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K8" s="11" t="s">
         <v>365</v>
@@ -9418,7 +9418,7 @@
         <v>24</v>
       </c>
       <c r="J6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>188</v>
@@ -9459,7 +9459,7 @@
         <v>573</v>
       </c>
       <c r="J7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K7" s="7" t="s">
         <v>188</v>
@@ -9500,7 +9500,7 @@
         <v>577</v>
       </c>
       <c r="J8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>188</v>
@@ -9579,7 +9579,7 @@
         <v>24</v>
       </c>
       <c r="J10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>188</v>
@@ -9620,7 +9620,7 @@
         <v>589</v>
       </c>
       <c r="J11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K11" s="7" t="s">
         <v>188</v>
@@ -9661,7 +9661,7 @@
         <v>589</v>
       </c>
       <c r="J12">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K12" s="7" t="s">
         <v>188</v>
@@ -9740,7 +9740,7 @@
         <v>24</v>
       </c>
       <c r="J14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K14" s="7" t="s">
         <v>188</v>
@@ -9781,7 +9781,7 @@
         <v>607</v>
       </c>
       <c r="J15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15" s="7" t="s">
         <v>188</v>
@@ -9860,7 +9860,7 @@
         <v>577</v>
       </c>
       <c r="J17">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K17" s="7" t="s">
         <v>188</v>
@@ -9901,7 +9901,7 @@
         <v>620</v>
       </c>
       <c r="J18">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K18" s="7" t="s">
         <v>188</v>
@@ -9942,7 +9942,7 @@
         <v>620</v>
       </c>
       <c r="J19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" s="7" t="s">
         <v>188</v>
@@ -9983,7 +9983,7 @@
         <v>620</v>
       </c>
       <c r="J20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="7" t="s">
         <v>188</v>
@@ -10110,8 +10110,12 @@
       <c r="I24" s="12" t="s">
         <v>620</v>
       </c>
-      <c r="J24" s="7"/>
-      <c r="K24" s="7"/>
+      <c r="J24">
+        <v>1</v>
+      </c>
+      <c r="K24" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L24" s="7" t="s">
         <v>645</v>
       </c>
@@ -10147,8 +10151,12 @@
       <c r="I25" s="7" t="s">
         <v>642</v>
       </c>
-      <c r="J25" s="7"/>
-      <c r="K25" s="7"/>
+      <c r="J25">
+        <v>1</v>
+      </c>
+      <c r="K25" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L25" s="7" t="s">
         <v>650</v>
       </c>
@@ -10184,8 +10192,12 @@
       <c r="I26" s="7" t="s">
         <v>647</v>
       </c>
-      <c r="J26" s="7"/>
-      <c r="K26" s="7"/>
+      <c r="J26">
+        <v>1</v>
+      </c>
+      <c r="K26" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L26" s="7" t="s">
         <v>654</v>
       </c>
@@ -10221,8 +10233,12 @@
       <c r="I27" s="7" t="s">
         <v>651</v>
       </c>
-      <c r="J27" s="7"/>
-      <c r="K27" s="7"/>
+      <c r="J27">
+        <v>1</v>
+      </c>
+      <c r="K27" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L27" s="7" t="s">
         <v>24</v>
       </c>
@@ -10258,8 +10274,12 @@
       <c r="I28" s="7" t="s">
         <v>655</v>
       </c>
-      <c r="J28" s="7"/>
-      <c r="K28" s="7"/>
+      <c r="J28">
+        <v>1</v>
+      </c>
+      <c r="K28" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L28" s="7" t="s">
         <v>24</v>
       </c>
@@ -10295,8 +10315,12 @@
       <c r="I29" s="7" t="s">
         <v>594</v>
       </c>
-      <c r="J29" s="7"/>
-      <c r="K29" s="7"/>
+      <c r="J29">
+        <v>1</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>188</v>
+      </c>
       <c r="L29" s="7" t="s">
         <v>600</v>
       </c>

</xml_diff>